<commit_message>
Update with latest result
</commit_message>
<xml_diff>
--- a/data/world_cup_2026.xlsx
+++ b/data/world_cup_2026.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Santanub\dev\fifa_2026\public\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CD44031D-7BE3-40A2-8D03-C609901CC262}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9C611289-AA65-4B16-80BD-BCFD325BA315}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="271" uniqueCount="137">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="274" uniqueCount="140">
   <si>
     <t>MatchID</t>
   </si>
@@ -437,6 +437,15 @@
   </si>
   <si>
     <t>Team 2 Yellow</t>
+  </si>
+  <si>
+    <t>Vinicious</t>
+  </si>
+  <si>
+    <t>Ismael</t>
+  </si>
+  <si>
+    <t>John McGinn</t>
   </si>
 </sst>
 </file>
@@ -967,14 +976,38 @@
       <c r="D7" t="s">
         <v>35</v>
       </c>
+      <c r="E7">
+        <v>1</v>
+      </c>
+      <c r="F7">
+        <v>1</v>
+      </c>
       <c r="G7" t="s">
         <v>8</v>
       </c>
       <c r="H7" t="s">
-        <v>36</v>
+        <v>21</v>
       </c>
       <c r="I7" t="s">
         <v>37</v>
+      </c>
+      <c r="J7" t="s">
+        <v>137</v>
+      </c>
+      <c r="K7" t="s">
+        <v>138</v>
+      </c>
+      <c r="L7">
+        <v>2</v>
+      </c>
+      <c r="M7">
+        <v>0</v>
+      </c>
+      <c r="N7">
+        <v>0</v>
+      </c>
+      <c r="O7">
+        <v>0</v>
       </c>
     </row>
     <row r="8" spans="1:15" x14ac:dyDescent="0.35">
@@ -990,14 +1023,35 @@
       <c r="D8" t="s">
         <v>39</v>
       </c>
+      <c r="E8">
+        <v>0</v>
+      </c>
+      <c r="F8">
+        <v>1</v>
+      </c>
       <c r="G8" t="s">
         <v>8</v>
       </c>
       <c r="H8" t="s">
-        <v>36</v>
+        <v>39</v>
       </c>
       <c r="I8" t="s">
         <v>37</v>
+      </c>
+      <c r="K8" t="s">
+        <v>139</v>
+      </c>
+      <c r="L8">
+        <v>1</v>
+      </c>
+      <c r="M8">
+        <v>3</v>
+      </c>
+      <c r="N8">
+        <v>0</v>
+      </c>
+      <c r="O8">
+        <v>0</v>
       </c>
     </row>
     <row r="9" spans="1:15" x14ac:dyDescent="0.35">

</xml_diff>

<commit_message>
few fixes and more deployment
</commit_message>
<xml_diff>
--- a/data/world_cup_2026.xlsx
+++ b/data/world_cup_2026.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Santanub\dev\fifa_2026\public\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9C611289-AA65-4B16-80BD-BCFD325BA315}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7E70B005-3B4D-4359-80EE-702CD2DEC24A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="274" uniqueCount="140">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="359" uniqueCount="141">
   <si>
     <t>MatchID</t>
   </si>
@@ -446,6 +446,9 @@
   </si>
   <si>
     <t>John McGinn</t>
+  </si>
+  <si>
+    <t>Columbia</t>
   </si>
 </sst>
 </file>
@@ -677,7 +680,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:O21"/>
+  <dimension ref="A1:O38"/>
   <sheetFormatPr defaultColWidth="8.58203125" defaultRowHeight="15.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="4" max="4" width="12.08203125" customWidth="1"/>
@@ -1351,6 +1354,397 @@
       </c>
       <c r="I21" t="s">
         <v>69</v>
+      </c>
+    </row>
+    <row r="22" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A22">
+        <v>21</v>
+      </c>
+      <c r="B22" s="1">
+        <v>46190</v>
+      </c>
+      <c r="C22" t="s">
+        <v>114</v>
+      </c>
+      <c r="D22" t="s">
+        <v>116</v>
+      </c>
+      <c r="G22" t="s">
+        <v>8</v>
+      </c>
+      <c r="H22" t="s">
+        <v>36</v>
+      </c>
+      <c r="I22" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="23" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A23">
+        <v>22</v>
+      </c>
+      <c r="B23" s="1">
+        <v>46191</v>
+      </c>
+      <c r="C23" t="s">
+        <v>101</v>
+      </c>
+      <c r="D23" t="s">
+        <v>105</v>
+      </c>
+      <c r="G23" t="s">
+        <v>8</v>
+      </c>
+      <c r="H23" t="s">
+        <v>36</v>
+      </c>
+      <c r="I23" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="24" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A24">
+        <v>23</v>
+      </c>
+      <c r="B24" s="1">
+        <v>46191</v>
+      </c>
+      <c r="C24" t="s">
+        <v>107</v>
+      </c>
+      <c r="D24" t="s">
+        <v>109</v>
+      </c>
+      <c r="G24" t="s">
+        <v>8</v>
+      </c>
+      <c r="H24" t="s">
+        <v>36</v>
+      </c>
+      <c r="I24" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="25" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A25">
+        <v>24</v>
+      </c>
+      <c r="B25" s="1">
+        <v>46191</v>
+      </c>
+      <c r="C25" t="s">
+        <v>118</v>
+      </c>
+      <c r="D25" t="s">
+        <v>140</v>
+      </c>
+      <c r="G25" t="s">
+        <v>8</v>
+      </c>
+      <c r="H25" t="s">
+        <v>36</v>
+      </c>
+      <c r="I25" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="26" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A26">
+        <v>25</v>
+      </c>
+      <c r="B26" s="1">
+        <v>46191</v>
+      </c>
+      <c r="C26" t="s">
+        <v>11</v>
+      </c>
+      <c r="D26" t="s">
+        <v>16</v>
+      </c>
+      <c r="G26" t="s">
+        <v>8</v>
+      </c>
+      <c r="H26" t="s">
+        <v>36</v>
+      </c>
+      <c r="I26" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="27" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A27">
+        <v>26</v>
+      </c>
+      <c r="B27" s="1">
+        <v>46192</v>
+      </c>
+      <c r="C27" t="s">
+        <v>20</v>
+      </c>
+      <c r="D27" t="s">
+        <v>31</v>
+      </c>
+      <c r="G27" t="s">
+        <v>8</v>
+      </c>
+      <c r="H27" t="s">
+        <v>36</v>
+      </c>
+      <c r="I27" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="28" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A28">
+        <v>27</v>
+      </c>
+      <c r="B28" s="1">
+        <v>46192</v>
+      </c>
+      <c r="C28" t="s">
+        <v>30</v>
+      </c>
+      <c r="D28" t="s">
+        <v>19</v>
+      </c>
+      <c r="G28" t="s">
+        <v>8</v>
+      </c>
+      <c r="H28" t="s">
+        <v>36</v>
+      </c>
+      <c r="I28" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="29" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A29">
+        <v>28</v>
+      </c>
+      <c r="B29" s="1">
+        <v>46192</v>
+      </c>
+      <c r="C29" t="s">
+        <v>15</v>
+      </c>
+      <c r="D29" t="s">
+        <v>12</v>
+      </c>
+      <c r="G29" t="s">
+        <v>8</v>
+      </c>
+      <c r="H29" t="s">
+        <v>36</v>
+      </c>
+      <c r="I29" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="30" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A30">
+        <v>29</v>
+      </c>
+      <c r="B30" s="1">
+        <v>46193</v>
+      </c>
+      <c r="C30" t="s">
+        <v>25</v>
+      </c>
+      <c r="D30" t="s">
+        <v>40</v>
+      </c>
+      <c r="G30" t="s">
+        <v>8</v>
+      </c>
+      <c r="H30" t="s">
+        <v>36</v>
+      </c>
+      <c r="I30" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="31" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A31">
+        <v>30</v>
+      </c>
+      <c r="B31" s="1">
+        <v>46193</v>
+      </c>
+      <c r="C31" t="s">
+        <v>39</v>
+      </c>
+      <c r="D31" t="s">
+        <v>35</v>
+      </c>
+      <c r="G31" t="s">
+        <v>8</v>
+      </c>
+      <c r="H31" t="s">
+        <v>36</v>
+      </c>
+      <c r="I31" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="32" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A32">
+        <v>31</v>
+      </c>
+      <c r="B32" s="1">
+        <v>46193</v>
+      </c>
+      <c r="C32" t="s">
+        <v>34</v>
+      </c>
+      <c r="D32" t="s">
+        <v>38</v>
+      </c>
+      <c r="G32" t="s">
+        <v>8</v>
+      </c>
+      <c r="H32" t="s">
+        <v>36</v>
+      </c>
+      <c r="I32" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="33" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A33">
+        <v>32</v>
+      </c>
+      <c r="B33" s="1">
+        <v>46193</v>
+      </c>
+      <c r="C33" t="s">
+        <v>41</v>
+      </c>
+      <c r="D33" t="s">
+        <v>26</v>
+      </c>
+      <c r="G33" t="s">
+        <v>8</v>
+      </c>
+      <c r="H33" t="s">
+        <v>36</v>
+      </c>
+      <c r="I33" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="34" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A34">
+        <v>33</v>
+      </c>
+      <c r="B34" s="1">
+        <v>46193</v>
+      </c>
+      <c r="C34" t="s">
+        <v>45</v>
+      </c>
+      <c r="D34" t="s">
+        <v>50</v>
+      </c>
+      <c r="G34" t="s">
+        <v>8</v>
+      </c>
+      <c r="H34" t="s">
+        <v>36</v>
+      </c>
+      <c r="I34" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="35" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A35">
+        <v>34</v>
+      </c>
+      <c r="B35" s="1">
+        <v>46194</v>
+      </c>
+      <c r="C35" t="s">
+        <v>42</v>
+      </c>
+      <c r="D35" t="s">
+        <v>48</v>
+      </c>
+      <c r="G35" t="s">
+        <v>8</v>
+      </c>
+      <c r="H35" t="s">
+        <v>36</v>
+      </c>
+      <c r="I35" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="36" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A36">
+        <v>35</v>
+      </c>
+      <c r="B36" s="1">
+        <v>46194</v>
+      </c>
+      <c r="C36" t="s">
+        <v>49</v>
+      </c>
+      <c r="D36" t="s">
+        <v>43</v>
+      </c>
+      <c r="G36" t="s">
+        <v>8</v>
+      </c>
+      <c r="H36" t="s">
+        <v>36</v>
+      </c>
+      <c r="I36" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="37" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A37">
+        <v>36</v>
+      </c>
+      <c r="B37" s="1">
+        <v>46194</v>
+      </c>
+      <c r="C37" t="s">
+        <v>51</v>
+      </c>
+      <c r="D37" t="s">
+        <v>46</v>
+      </c>
+      <c r="G37" t="s">
+        <v>8</v>
+      </c>
+      <c r="H37" t="s">
+        <v>36</v>
+      </c>
+      <c r="I37" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="38" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A38">
+        <v>37</v>
+      </c>
+      <c r="B38" s="1">
+        <v>46194</v>
+      </c>
+      <c r="C38" t="s">
+        <v>52</v>
+      </c>
+      <c r="D38" t="s">
+        <v>58</v>
+      </c>
+      <c r="G38" t="s">
+        <v>8</v>
+      </c>
+      <c r="H38" t="s">
+        <v>36</v>
+      </c>
+      <c r="I38" t="s">
+        <v>54</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat: release few new changes
</commit_message>
<xml_diff>
--- a/data/world_cup_2026.xlsx
+++ b/data/world_cup_2026.xlsx
@@ -18,7 +18,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="716" uniqueCount="187">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="915" uniqueCount="305">
   <si>
     <t>MatchID</t>
   </si>
@@ -203,9 +203,6 @@
     <t>Ecuador</t>
   </si>
   <si>
-    <t xml:space="preserve">Ecuador </t>
-  </si>
-  <si>
     <t>Diallo</t>
   </si>
   <si>
@@ -239,193 +236,553 @@
     <t>G</t>
   </si>
   <si>
+    <t>Hany(OG)</t>
+  </si>
+  <si>
+    <t>Ashour</t>
+  </si>
+  <si>
+    <t>Saudi Arabia</t>
+  </si>
+  <si>
+    <t>Uruguay</t>
+  </si>
+  <si>
+    <t>Amri</t>
+  </si>
+  <si>
+    <t>Araujo</t>
+  </si>
+  <si>
+    <t>Iran</t>
+  </si>
+  <si>
+    <t>New Zealand</t>
+  </si>
+  <si>
+    <t>Rezaeian, Mohebi</t>
+  </si>
+  <si>
+    <t>E Just , E Just</t>
+  </si>
+  <si>
+    <t>France</t>
+  </si>
+  <si>
+    <t>Senegal</t>
+  </si>
+  <si>
+    <t>I</t>
+  </si>
+  <si>
+    <t>Mbappe, Barcola, Mbappe</t>
+  </si>
+  <si>
+    <t>Mbaye</t>
+  </si>
+  <si>
+    <t>Iraq</t>
+  </si>
+  <si>
+    <t>Norway</t>
+  </si>
+  <si>
+    <t>Hussein</t>
+  </si>
+  <si>
+    <t>Haaland, Haaland, Ostigard, Hussein(OG)</t>
+  </si>
+  <si>
+    <t>Argentina</t>
+  </si>
+  <si>
+    <t>Algeria</t>
+  </si>
+  <si>
+    <t>J</t>
+  </si>
+  <si>
+    <t>Messi, Messi, Messi</t>
+  </si>
+  <si>
+    <t>Austria</t>
+  </si>
+  <si>
+    <t>Jordon</t>
+  </si>
+  <si>
+    <t>Romano Schimd, Marko Arnautovic, Yazan Al-Arab(OG)</t>
+  </si>
+  <si>
+    <t>Ali Olwan</t>
+  </si>
+  <si>
+    <t>Portugal</t>
+  </si>
+  <si>
+    <t>DR Congo</t>
+  </si>
+  <si>
+    <t>K</t>
+  </si>
+  <si>
+    <t>Neves</t>
+  </si>
+  <si>
+    <t>Wissa</t>
+  </si>
+  <si>
+    <t>England</t>
+  </si>
+  <si>
+    <t>Croatia</t>
+  </si>
+  <si>
+    <t>L</t>
+  </si>
+  <si>
+    <t>Harry Kane, Harry Kane, Bellingham, Rashford</t>
+  </si>
+  <si>
+    <t>Baturina, Peter Musa</t>
+  </si>
+  <si>
+    <t>Ghana</t>
+  </si>
+  <si>
+    <t>Panama</t>
+  </si>
+  <si>
+    <t>Yirenkyi</t>
+  </si>
+  <si>
+    <t>Uzbekistan</t>
+  </si>
+  <si>
+    <t>Columbia</t>
+  </si>
+  <si>
+    <t>Abbosbek Fayzullaev</t>
+  </si>
+  <si>
+    <t>Daniel Munoz, Luis Diaz, Jaminton Campaz</t>
+  </si>
+  <si>
+    <t>Mokoena</t>
+  </si>
+  <si>
+    <t>Sadilek</t>
+  </si>
+  <si>
+    <t>Ermin Mahmic</t>
+  </si>
+  <si>
+    <t>Johan Manzambi, Ruben Vargas, Johan Manzambi, Xhaka</t>
+  </si>
+  <si>
+    <t>Cyle Larin, Jonathan David, Jonathan David, Saliba, Manai(OG), Jonathan David</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mexico </t>
+  </si>
+  <si>
+    <t>Luis Romo</t>
+  </si>
+  <si>
+    <t>TBD</t>
+  </si>
+  <si>
+    <t>Jordan</t>
+  </si>
+  <si>
+    <t>Round of 32</t>
+  </si>
+  <si>
+    <t>Round of 16</t>
+  </si>
+  <si>
+    <t>Quarter-finals</t>
+  </si>
+  <si>
+    <t>Semi-finals</t>
+  </si>
+  <si>
+    <t>Third place</t>
+  </si>
+  <si>
+    <t>Final</t>
+  </si>
+  <si>
+    <t>Player Name</t>
+  </si>
+  <si>
+    <t>Country</t>
+  </si>
+  <si>
+    <t>Image</t>
+  </si>
+  <si>
+    <t>Jullan</t>
+  </si>
+  <si>
+    <t>https://media.bolavip.com/wp-content/uploads/sites/10/2026/06/11153815/Julian-Quinones-1-1200x740.webp</t>
+  </si>
+  <si>
+    <t>Raul</t>
+  </si>
+  <si>
+    <t>https://upload.wikimedia.org/wikipedia/commons/thumb/d/de/Ra%C3%BAl_Jim%C3%A9nez_04032026_%281%29.jpg/250px-Ra%C3%BAl_Jim%C3%A9nez_04032026_%281%29.jpg</t>
+  </si>
+  <si>
+    <t>Hawang in-beom</t>
+  </si>
+  <si>
+    <t>https://upload.wikimedia.org/wikipedia/commons/thumb/8/8e/240611_%EB%8C%80%ED%95%9C%EB%AF%BC%EA%B5%AD_vs_%EC%A4%91%EA%B5%AD_%28%ED%99%A9%EC%9D%B8%EB%B2%94%29.jpg/250px-240611_%EB%8C%80%ED%95%9C%EB%AF%BC%EA%B5%AD_vs_%EC%A4%91%EA%B5%AD_%28%ED%99%A9%EC%9D%B8%EB%B2%94%29.jpg</t>
+  </si>
+  <si>
+    <t>Hyeon-gyu</t>
+  </si>
+  <si>
+    <t>https://upload.wikimedia.org/wikipedia/commons/thumb/b/b4/Oh_Hyeon-gyu_BJK.jpeg/250px-Oh_Hyeon-gyu_BJK.jpeg</t>
+  </si>
+  <si>
+    <t>https://media.gettyimages.com/id/2281158964/photo/guadalajara-mexico-ladislav-krejci-of-czechia-celebrates-scoring-his-teams-first-goal-during.jpg?s=612x612&amp;w=gi&amp;k=20&amp;c=6wh-hBwkWJaUmM0dxx9svMRbSngWMFB6ESBcKfDVZ3o=</t>
+  </si>
+  <si>
+    <t>https://www.vmcdn.ca/f/files/shared/feeds/cp/2021/05/20210501160528-608dba988b3294a3bef8930bjpeg.jpg</t>
+  </si>
+  <si>
+    <t>https://encrypted-tbn0.gstatic.com/images?q=tbn:ANd9GcQNMb-COzX-f0jgiosmYJWhnzqnyOCjj2lsbw&amp;s</t>
+  </si>
+  <si>
+    <t>Damian Bobadilla</t>
+  </si>
+  <si>
+    <t>https://encrypted-tbn1.gstatic.com/licensed-image?q=tbn:ANd9GcRSD0yqwgntMLnleRin-4fYCXZ5IoIw4ene59lVt_ljRbQ4Xj2T33oxJ4Xotv8L5HC6y8JtBUVZGvqA-VQ</t>
+  </si>
+  <si>
+    <t>https://encrypted-tbn0.gstatic.com/images?q=tbn:ANd9GcRKRAKs7r3G0uPX2cTrYzcg0BlM76ozOLItew&amp;s</t>
+  </si>
+  <si>
+    <t>Giovanni Reyna</t>
+  </si>
+  <si>
+    <t>https://www.usanetwork.com/sites/usablog/files/2022/12/world-cup-gio-reyna.jpg</t>
+  </si>
+  <si>
+    <t>Folarin Balogun</t>
+  </si>
+  <si>
+    <t>https://assets.goal.com/images/v3/blt62467338dffc08d5/balogun.jpg</t>
+  </si>
+  <si>
+    <t>https://upload.wikimedia.org/wikipedia/commons/thumb/5/55/Boualem_Khoukhi.png/250px-Boualem_Khoukhi.png</t>
+  </si>
+  <si>
+    <t>https://ichef.bbci.co.uk/ace/standard/1920/cpsprodpb/f186/live/1124bab0-6061-11f1-8194-8105d46fb81b.jpg</t>
+  </si>
+  <si>
+    <t>Messi</t>
+  </si>
+  <si>
+    <t>https://upload.wikimedia.org/wikipedia/commons/1/18/Lionel-Messi-Argentina-2022-FIFA-World-Cup_sharpness.jpg</t>
+  </si>
+  <si>
+    <t>https://jordantimes.com/jordantimes/uploads/images/2025/12/31/709442.webp</t>
+  </si>
+  <si>
+    <t>Romano Schimd</t>
+  </si>
+  <si>
+    <t>https://encrypted-tbn3.gstatic.com/licensed-image?q=tbn:ANd9GcTmLc8iLqRGpdVuwd22ONVsH7Kuyw6xv23yorz4Zd5cv4Yv19GF8g5WJNtAB0_5EN_5NcuBqq9jelqBF60</t>
+  </si>
+  <si>
+    <t>Marko Arnautovic</t>
+  </si>
+  <si>
+    <t>https://encrypted-tbn0.gstatic.com/images?q=tbn:ANd9GcQZjddLOrCZRBd0UgAD6eRWMzqFZNuJRWAtroQ9B3GC8balofT0i-AMYvSYbbBj9Ba-yQG3T_Tbt5aM_77yLQwDlKqedIsRhf9VnGohGQ&amp;s=10</t>
+  </si>
+  <si>
+    <t>Yazan Al-Arab</t>
+  </si>
+  <si>
+    <t>https://encrypted-tbn3.gstatic.com/licensed-image?q=tbn:ANd9GcS-n6J3Xtx65uWHKqkIyV7MBn4PeHm24sm-Ei8qmQTXIS0GXKR3aLn6C-OEOW9uuIH0UTZJ6YAZAEuDHsc</t>
+  </si>
+  <si>
+    <t>https://encrypted-tbn1.gstatic.com/licensed-image?q=tbn:ANd9GcSdPfCz7MI_tDXuQ6lqhobcSQyuaGP7tYFQUMXFZYTDViW5U39dZ58QM9ZCelp6JUjQHHqP157sQSZVkwo</t>
+  </si>
+  <si>
+    <t>https://upload.wikimedia.org/wikipedia/commons/thumb/b/b5/Ismael_Saibari_Morocco_v_Norway_7_June_2026-162_%28cropped%29.jpg/250px-Ismael_Saibari_Morocco_v_Norway_7_June_2026-162_%28cropped%29.jpg</t>
+  </si>
+  <si>
+    <t>https://encrypted-tbn1.gstatic.com/licensed-image?q=tbn:ANd9GcTdaBYFK_lw1pHJDWE81Sq5k0R7EVuV4y5rWRnCrH_3IImi-1iXAygnRdGmnrjJW1omMPwEKnxTUCWk0rk</t>
+  </si>
+  <si>
+    <t>Nestroy</t>
+  </si>
+  <si>
+    <t>https://encrypted-tbn1.gstatic.com/licensed-image?q=tbn:ANd9GcRjVQ5djADnBnswHLwtP7bQ1TI3Rryq_CGyYsqRPayyJPVYxzs7foMm3KzslU5j-XOew9ZwrZ4ZZ2kgHW8</t>
+  </si>
+  <si>
+    <t>Connor Metacalfe</t>
+  </si>
+  <si>
+    <t>https://encrypted-tbn0.gstatic.com/images?q=tbn:ANd9GcSgygN-KzKvlTRXg-8pRQrMd_F2IPG5OBFqyarNygjleb0uTUydB-hv6L-J4HL5yYao2p6X8yXosKkGDcwiLyiBMyOvNTVwczqsWFPi83E&amp;s=10</t>
+  </si>
+  <si>
+    <t>Nmecha</t>
+  </si>
+  <si>
+    <t>https://encrypted-tbn3.gstatic.com/licensed-image?q=tbn:ANd9GcQYqlFmucCAC3W-Al-ZeCIisZUNF7A62ONWmXZMkUe0sGUbMfE5YmJeGUR4fUSZ4O8yf8DJjTyAK1Q2Vxc</t>
+  </si>
+  <si>
+    <t>Havertz</t>
+  </si>
+  <si>
+    <t>https://encrypted-tbn2.gstatic.com/licensed-image?q=tbn:ANd9GcSw8zr1JoFSnF8QHU9vDO2zUcCYNrg8w4s6yR3o0ZXqY8lBofb5FyMfSB4sGEhkL9dcZfGxLyTYHGbCTbU</t>
+  </si>
+  <si>
+    <t>Undav</t>
+  </si>
+  <si>
+    <t>https://encrypted-tbn0.gstatic.com/licensed-image?q=tbn:ANd9GcT7DlrM_OYHSJ-dl70RTcEL-QknaTR-N0QG7gRFY8J1Ub27Ir1lqDawL7ax7AhKeq2UZgCbZqBiht7jTIwROvom581ja5o3qLntOkHwLLwRZqqzT2-mpdSbIDnN2gAGvdjP2h-XRuSk1A&amp;s=19</t>
+  </si>
+  <si>
+    <t>Brown</t>
+  </si>
+  <si>
+    <t>https://encrypted-tbn0.gstatic.com/licensed-image?q=tbn:ANd9GcTy7hc26D6Kp4oDzYNj_H3SsIwQQPEFOPOT05dAoBa5gPFxsZRIKxp4Pa2ZiiJbQgtJvpwe_xCVdtrPlDQ</t>
+  </si>
+  <si>
+    <t>Musiala</t>
+  </si>
+  <si>
+    <t>https://encrypted-tbn0.gstatic.com/images?q=tbn:ANd9GcR5VLvgh0N2AKR9GdsRWiyM5BoSNfPS9n8UEjnQMuP8XkNTJ118tyCufRXBOX2n6lk-Uibrs3NC4p_PE_GAV_nZt-vtN7ppP4rdZu4xVw&amp;s=10</t>
+  </si>
+  <si>
+    <t>Schlotterbake</t>
+  </si>
+  <si>
+    <t>https://assets.goal.com/images/v3/blt95ffc0239096ec4c/Nico%20Schlotterbeck%20Germany%202024%20(2).jpg?auto=webp&amp;format=pjpg&amp;width=3840&amp;quality=60</t>
+  </si>
+  <si>
+    <t>https://encrypted-tbn3.gstatic.com/licensed-image?q=tbn:ANd9GcSOtBK_Kp-xjuOpZzdqswB36km5ZbN9H6irAbg0bMipboJhAo9QiVw6VMeH0wD1Tk3zfj7EUL_GnVSwoX0</t>
+  </si>
+  <si>
+    <t>Dijk</t>
+  </si>
+  <si>
+    <t>https://encrypted-tbn3.gstatic.com/licensed-image?q=tbn:ANd9GcSRlnqqOmWI5DTrHNs8kxZBo4N0_Idr01UTD-IrDc0sZAPo6oMJpjw57qu88tXqj4ZsgdypJk_6FsniUdM</t>
+  </si>
+  <si>
+    <t>Nakamura</t>
+  </si>
+  <si>
+    <t>https://encrypted-tbn1.gstatic.com/licensed-image?q=tbn:ANd9GcQgSs3ZltwYtUvka9BBcA-U5wiOkAgKU7jkzJQwBa7_9v_VnUf4tva3P8j0WUQgtNW6VAt5HlHX1NsHS8U</t>
+  </si>
+  <si>
+    <t>Kamada</t>
+  </si>
+  <si>
+    <t>https://encrypted-tbn1.gstatic.com/licensed-image?q=tbn:ANd9GcQiPOESRcnY9oq92s_7KO7FfRlH7wVPofyua9JWb9-ozuMZ8P-HXF02KX9DOhBPzzGU8Z9KwUG1yTYtDKs</t>
+  </si>
+  <si>
+    <t>Summervile</t>
+  </si>
+  <si>
+    <t>https://encrypted-tbn2.gstatic.com/licensed-image?q=tbn:ANd9GcQkUnzg_gSnBrdW666MqkIh9Qf6CFZsXpQFu7T7PZOkOTimlIj7yuE0lj64Quxz8x1_GaIb899HCDUjdm0</t>
+  </si>
+  <si>
+    <t>https://encrypted-tbn0.gstatic.com/images?q=tbn:ANd9GcRWwc36OuYWwlgCH1G5GDg01I4zB9BlSisyQg&amp;s</t>
+  </si>
+  <si>
+    <t>Yasin Ayari</t>
+  </si>
+  <si>
+    <t>https://im.rediff.com/sports/2026/jun/15ayari1.jpg?w=670&amp;h=900</t>
+  </si>
+  <si>
+    <t>https://encrypted-tbn2.gstatic.com/licensed-image?q=tbn:ANd9GcTWBHRSGDjHVWxfS3c5Z_rhWUfYdeVjcuOeHrBJz9kt6jAtGGuhU_mqhOLcKl4tTaP6AhMnd_VxZhF-DVI</t>
+  </si>
+  <si>
+    <t>Mattias</t>
+  </si>
+  <si>
+    <t>https://www.hindustantimes.com/ht-img/img/2026/06/15/550x309/SOCCER-WORLDCUP-SWE-TUN--260_1781514642061_1781514661109_37b9e4ac-fd22-459a-b250-c0c24278d9bd.JPG</t>
+  </si>
+  <si>
+    <t>Viktor Gyökeres</t>
+  </si>
+  <si>
+    <t>https://i.guim.co.uk/img/media/27b82fe812ed12e57bf6bcabb32d91515328f99d/0_362_5682_3409/master/5682.jpg?width=1200&amp;quality=85&amp;auto=format&amp;fit=max&amp;s=6dd8dae8f08fef77b5db3d20e38e16d3</t>
+  </si>
+  <si>
+    <t>Alexander Isak</t>
+  </si>
+  <si>
+    <t>https://ichef.bbci.co.uk/ace/standard/699/cpsprodpb/48b9/live/ebd59b50-8337-11f0-8ded-85867f31a902.jpg</t>
+  </si>
+  <si>
     <t>Hany</t>
   </si>
   <si>
-    <t>Ashour</t>
-  </si>
-  <si>
-    <t>Saudi Arabia</t>
-  </si>
-  <si>
-    <t>Uruguay</t>
-  </si>
-  <si>
-    <t>Amri</t>
-  </si>
-  <si>
-    <t>Araujo</t>
-  </si>
-  <si>
-    <t>Iran</t>
-  </si>
-  <si>
-    <t>New Zealand</t>
-  </si>
-  <si>
-    <t>Rezaeian, Mohebi</t>
-  </si>
-  <si>
-    <t>E Just , E Just</t>
-  </si>
-  <si>
-    <t>France</t>
-  </si>
-  <si>
-    <t>Senegal</t>
-  </si>
-  <si>
-    <t>I</t>
-  </si>
-  <si>
-    <t>Mbappe, Barcola, Mbappe</t>
-  </si>
-  <si>
-    <t>Mbaye</t>
-  </si>
-  <si>
-    <t>Iraq</t>
-  </si>
-  <si>
-    <t>Norway</t>
-  </si>
-  <si>
-    <t>Hussein</t>
-  </si>
-  <si>
-    <t>Haaland, Haaland, Ostigard, Hussein(OG)</t>
-  </si>
-  <si>
-    <t>Argentina</t>
-  </si>
-  <si>
-    <t>Algeria</t>
-  </si>
-  <si>
-    <t>J</t>
-  </si>
-  <si>
-    <t>Messi, Messi, Messi</t>
-  </si>
-  <si>
-    <t>Austria</t>
-  </si>
-  <si>
-    <t>Jordon</t>
-  </si>
-  <si>
-    <t>TBD</t>
-  </si>
-  <si>
-    <t>Portugal</t>
-  </si>
-  <si>
-    <t>DR Congo</t>
-  </si>
-  <si>
-    <t>K</t>
-  </si>
-  <si>
-    <t>England</t>
-  </si>
-  <si>
-    <t>Croatia</t>
-  </si>
-  <si>
-    <t>L</t>
-  </si>
-  <si>
-    <t>Ghana</t>
-  </si>
-  <si>
-    <t>Panama</t>
-  </si>
-  <si>
-    <t>Uzbekistan</t>
-  </si>
-  <si>
-    <t>Columbia</t>
-  </si>
-  <si>
-    <t>Jordan</t>
-  </si>
-  <si>
-    <t>Round of 32</t>
-  </si>
-  <si>
-    <t>Round of 16</t>
-  </si>
-  <si>
-    <t>Quarter-finals</t>
-  </si>
-  <si>
-    <t>Semi-finals</t>
-  </si>
-  <si>
-    <t>Third place</t>
-  </si>
-  <si>
-    <t>Final</t>
-  </si>
-  <si>
-    <t>Player Name</t>
-  </si>
-  <si>
-    <t>Country</t>
-  </si>
-  <si>
-    <t>Image</t>
-  </si>
-  <si>
-    <t>Jullan</t>
-  </si>
-  <si>
-    <t>https://media.bolavip.com/wp-content/uploads/sites/10/2026/06/11153815/Julian-Quinones-1-1200x740.webp</t>
-  </si>
-  <si>
-    <t>Raul</t>
-  </si>
-  <si>
-    <t>https://upload.wikimedia.org/wikipedia/commons/thumb/d/de/Ra%C3%BAl_Jim%C3%A9nez_04032026_%281%29.jpg/250px-Ra%C3%BAl_Jim%C3%A9nez_04032026_%281%29.jpg</t>
-  </si>
-  <si>
-    <t>Hawang in-beom</t>
-  </si>
-  <si>
-    <t>https://upload.wikimedia.org/wikipedia/commons/thumb/8/8e/240611_%EB%8C%80%ED%95%9C%EB%AF%BC%EA%B5%AD_vs_%EC%A4%91%EA%B5%AD_%28%ED%99%A9%EC%9D%B8%EB%B2%94%29.jpg/250px-240611_%EB%8C%80%ED%95%9C%EB%AF%BC%EA%B5%AD_vs_%EC%A4%91%EA%B5%AD_%28%ED%99%A9%EC%9D%B8%EB%B2%94%29.jpg</t>
-  </si>
-  <si>
-    <t>Hyeon-gyu</t>
-  </si>
-  <si>
-    <t>https://upload.wikimedia.org/wikipedia/commons/thumb/b/b4/Oh_Hyeon-gyu_BJK.jpeg/250px-Oh_Hyeon-gyu_BJK.jpeg</t>
-  </si>
-  <si>
-    <t>https://media.gettyimages.com/id/2281158964/photo/guadalajara-mexico-ladislav-krejci-of-czechia-celebrates-scoring-his-teams-first-goal-during.jpg?s=612x612&amp;w=gi&amp;k=20&amp;c=6wh-hBwkWJaUmM0dxx9svMRbSngWMFB6ESBcKfDVZ3o=</t>
-  </si>
-  <si>
-    <t>https://www.vmcdn.ca/f/files/shared/feeds/cp/2021/05/20210501160528-608dba988b3294a3bef8930bjpeg.jpg</t>
-  </si>
-  <si>
-    <t>https://encrypted-tbn0.gstatic.com/images?q=tbn:ANd9GcQNMb-COzX-f0jgiosmYJWhnzqnyOCjj2lsbw&amp;s</t>
-  </si>
-  <si>
-    <t>Damian Bobadilla</t>
-  </si>
-  <si>
-    <t>https://encrypted-tbn0.gstatic.com/images?q=tbn:ANd9GcRKRAKs7r3G0uPX2cTrYzcg0BlM76ozOLItew&amp;s</t>
-  </si>
-  <si>
-    <t>Giovanni Reyna</t>
-  </si>
-  <si>
-    <t>https://www.usanetwork.com/sites/usablog/files/2022/12/world-cup-gio-reyna.jpg</t>
-  </si>
-  <si>
-    <t>Folarin Balogun</t>
-  </si>
-  <si>
-    <t>https://assets.goal.com/images/v3/blt62467338dffc08d5/balogun.jpg</t>
+    <t>https://encrypted-tbn0.gstatic.com/licensed-image?q=tbn:ANd9GcRJvUQELUfyfES8w9_bs0o1cuzMOHO2Lpi3UXdjpY7UYiO9YbwFSWS1T-wYRbdPONv5U-5Z8DHQ38z9rgk</t>
+  </si>
+  <si>
+    <t>https://encrypted-tbn0.gstatic.com/licensed-image?q=tbn:ANd9GcQtUuj_nhddI7aOwmEjkxtk9eBvBrd2kb8b37FQJcpOFQg2-AY12rbaLKlPp6CqpLJSihi81pJ0lrhwbi4</t>
+  </si>
+  <si>
+    <t>https://encrypted-tbn0.gstatic.com/images?q=tbn:ANd9GcR3z8DSDg58ww1Su5qTuNST61NRy7y6hyfEM0IxBjEWLDo_72QtCqxXDPR1kilyu6jLMKjvcrU_Re58-q1SDtb8BOgCUC5SyTTJukdzomI&amp;s=10</t>
+  </si>
+  <si>
+    <t>https://encrypted-tbn0.gstatic.com/images?q=tbn:ANd9GcRezkA8KBy8ve1i6vzA-0QVUiXh_zkgitdV6OT5PvJlpRL1AR31XSXk-ZVP8ktc-3C6YiW2nk1G8eJhiDLhusk-fZJ2P5UkAIpemcEZOC0&amp;s=10</t>
+  </si>
+  <si>
+    <t>Rezaeian</t>
+  </si>
+  <si>
+    <t>https://encrypted-tbn0.gstatic.com/images?q=tbn:ANd9GcT81PXvNo5X5RMU2mbxdTqH-Lv2vXXbrwlqBeN5j2LjSNSGLNLPfS-2h3RgFObfOLeGb9aLzHhCIZol3mXLD5Y1zA5I4djATY1m6QaQcw&amp;s=10</t>
+  </si>
+  <si>
+    <t>E Just</t>
+  </si>
+  <si>
+    <t>https://encrypted-tbn1.gstatic.com/licensed-image?q=tbn:ANd9GcSvLKGPfOmyh_EvJM73aiRZuSRzMBitX48UyiH-FnCWhTfFcTnpZwHfzlPspzgENVFDxwGKz4HWj_iWEqg</t>
+  </si>
+  <si>
+    <t>Mohebi</t>
+  </si>
+  <si>
+    <t>https://encrypted-tbn0.gstatic.com/images?q=tbn:ANd9GcTzIJ54mDvzZCVHp0Gnm8MOoYHwwcCjWjkl5lN-hyAssHKOFD5FdoYLhppmfoXdGPJpQUKA8ize5cwEdyduEDrjMLgXeg2S7j4a-o3FfjI&amp;s=10</t>
+  </si>
+  <si>
+    <t>Mbappe</t>
+  </si>
+  <si>
+    <t>https://assets.goal.com/images/v3/blt4eee8b74938714db/mbappe-france-16-9.jpg?auto=webp&amp;format=pjpg&amp;width=3840&amp;quality=60</t>
+  </si>
+  <si>
+    <t>https://encrypted-tbn1.gstatic.com/licensed-image?q=tbn:ANd9GcTzUq0JJSefIvZtJ8UtAzj5X6KHsWbfgVpbCfZPBQn75Yl22r3B_m_pNP03f0TXOTOXXrsbpusVyXXpCF8</t>
+  </si>
+  <si>
+    <t>Barcola</t>
+  </si>
+  <si>
+    <t>https://encrypted-tbn0.gstatic.com/licensed-image?q=tbn:ANd9GcSNIQCMW0hkQ_tGMymRe_W3flCRRoAqs3qtC3ajJDZ9IWKOCKi6A9BgYDbJaI8V2TmF81iHBJP0_5rxaZM</t>
+  </si>
+  <si>
+    <t>https://media.openthemagazine.com/openthemagazine/2026-06-17/9wkod8fu/Aymen-Hussain.jpg?w=640&amp;auto=format,compress&amp;q=80</t>
+  </si>
+  <si>
+    <t>Haaland</t>
+  </si>
+  <si>
+    <t>https://encrypted-tbn0.gstatic.com/licensed-image?q=tbn:ANd9GcS2ZrfE2QdOBZqm23pcR4F8y9bSO_tZ0Vuky6B-cD-viBG-cgfR-Aa2f0IZ36TuNexHk8O8QNXERis_pdU</t>
+  </si>
+  <si>
+    <t>Ostigard</t>
+  </si>
+  <si>
+    <t>https://encrypted-tbn0.gstatic.com/licensed-image?q=tbn:ANd9GcR_c1eJ1p_9Y7lS2SN7J6_cj00Yz8yHv721D7SjCdpXB1ro4XwZy7TSua5jGTs_7om2xUbqpGTGAj8gaus</t>
+  </si>
+  <si>
+    <t>https://encrypted-tbn0.gstatic.com/licensed-image?q=tbn:ANd9GcRmjcrYnsKo0tY2rG2gdjN6dNfT9Y0wHBE2UP8xJeax0wIR7xh08J2VWDAUay-NwPFEIg2CBRoV-7Lu__MR9bBWwjtrVlq0eHhPsvwMD-KpvcMJXSr5W2mzasLtcMP6HEuq9lZA77LBKeNT&amp;s=19</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Portugal </t>
+  </si>
+  <si>
+    <t>https://encrypted-tbn0.gstatic.com/images?q=tbn:ANd9GcSFHXgRvzq545VRSGjUk_W8qpz4o01xfdvHDNTZJmNVDUykrbaDOKPz0nq_ce3TKjMtXnMJKDraO36Ub6xKP5iyzA8gwjmBd8TZ_RwsOEcJ&amp;s=10</t>
+  </si>
+  <si>
+    <t>Baturina</t>
+  </si>
+  <si>
+    <t>https://encrypted-tbn3.gstatic.com/licensed-image?q=tbn:ANd9GcSjCywA5x2IcU_Bz5qk0-ttE_iVAzFSqoOGd7hCkXNalZzS4RVPeua9JfEyGG5DV8r4Zfmi-Ljq9yPI5oE</t>
+  </si>
+  <si>
+    <t>Peter Musa</t>
+  </si>
+  <si>
+    <t>https://encrypted-tbn1.gstatic.com/licensed-image?q=tbn:ANd9GcQye6N91wHZIZUk-EUpqWNdazCQjsIMzPaqLJqeZHsLvv52w8XL0wPKmi0bZbs5iwqGZChv8yK2Qk8pA1c</t>
+  </si>
+  <si>
+    <t>Harry Kane</t>
+  </si>
+  <si>
+    <t>https://encrypted-tbn2.gstatic.com/licensed-image?q=tbn:ANd9GcQ-d1g0QLbd79gWMtX4Ij5blDshR6SdMx-K0G0K9SAKvXa2zSns2GGFOlzcoi8QnAewAJGSB6qjS1WjEEI</t>
+  </si>
+  <si>
+    <t>Rashford</t>
+  </si>
+  <si>
+    <t>https://encrypted-tbn1.gstatic.com/licensed-image?q=tbn:ANd9GcTQDNfr38sykErOwZ6Yb7E1wFr1gONaC5DmBvCd36hdgqx4IiYaYc1b3mCn90tQ4QuoUzrGMW-qGFKLBM4</t>
+  </si>
+  <si>
+    <t>Bellingham</t>
+  </si>
+  <si>
+    <t>https://encrypted-tbn1.gstatic.com/licensed-image?q=tbn:ANd9GcSYIfC0zxZp5w3nhcgn_tev69AcXi96ZtJ1roi7OSYHwnScx0UuCCKKQ4_WnmmnPvBLSgHg2SW0NkCCGas</t>
+  </si>
+  <si>
+    <t>https://encrypted-tbn0.gstatic.com/licensed-image?q=tbn:ANd9GcRIFh6-iuUllHoBiQNWgv-EMUq0bFwayg4ZycxUZqBKzV0MCivLw2MAQEEw7XJSn_PqQTo10kXzPc3R3Z3t8SfyOnASUPyqLBQM_ovyILqxHDpFyz9g3xKgtOWt_zgZ7TNbLIR9OXuhrA&amp;s=19</t>
+  </si>
+  <si>
+    <t>Daniel Munoz</t>
+  </si>
+  <si>
+    <t>https://encrypted-tbn3.gstatic.com/licensed-image?q=tbn:ANd9GcQiE2EzwIXfaSvsXMYkp0a0895aCN2LsL1u1JvBrXjmxbQTRr8x3RRyFFGD3lmg_fp39T7gpD35twhWyeo</t>
+  </si>
+  <si>
+    <t>Luis Diaz</t>
+  </si>
+  <si>
+    <t>https://encrypted-tbn0.gstatic.com/images?q=tbn:ANd9GcQPfJ6GPMr9fnlxRqwwXCbmOZMaXqZqbesCghiJHYp_FnnBnJH1vWQ4d3JjlT7AFx2NDT5LKREJv2YolqIQni-KR2c7RcWq07iyuXvPIA&amp;s=10</t>
+  </si>
+  <si>
+    <t>Jaminton Campaz</t>
+  </si>
+  <si>
+    <t>https://encrypted-tbn0.gstatic.com/licensed-image?q=tbn:ANd9GcRYzQox5_qWjlAIrVd2FWSL9bBRCfDr3ky-V8bHXRQi3ph5yxxKmb_5CLxnhM4PuJFcH6V0fE4vXhvVn7c</t>
+  </si>
+  <si>
+    <t>https://ichef.bbci.co.uk/ace/standard/1920/cpsprodpb/91f4/live/e0b99250-264d-11ef-aca4-1d72b2f67b66.jpg</t>
+  </si>
+  <si>
+    <t>https://encrypted-tbn0.gstatic.com/images?q=tbn:ANd9GcRhaIu7yp0X5nMNB6sgrXWXDw4CSYoRws8-BS3m5hqXDc_ZymRYtDyvLXKanlBTgoWym-mqi09PRJP7ahoGxVSxHr4_lewGv1eSccZtdQ&amp;s=10</t>
+  </si>
+  <si>
+    <t>https://encrypted-tbn0.gstatic.com/images?q=tbn:ANd9GcR5F3sD-0qO_MxCwpBK4TSm7XK78bdfq-GDRGBz0RuduWzmxF0nBzAzDacpdUrFOUG4WXvcPOoOamPvF1y0MpLEOnzrw4zna0uPOkE2ab90fw&amp;s=10</t>
+  </si>
+  <si>
+    <t>Johan Manzambi</t>
+  </si>
+  <si>
+    <t>https://encrypted-tbn0.gstatic.com/images?q=tbn:ANd9GcQjB2i2QEHZKnfRZpHlGJGD4dSyNIzRhFU1s8F-gkEC573zEM7sDzTSxdGTGVdo0NFpY132TvGaf85HOke7LUWwthU4yTy_0ETahgKbpUbZ&amp;s=10</t>
+  </si>
+  <si>
+    <t>Ruben Vargas</t>
+  </si>
+  <si>
+    <t>https://encrypted-tbn3.gstatic.com/licensed-image?q=tbn:ANd9GcRuC7ZT4NueP40JgwSDyi_PFYz46CVSHNn7qvKiOqsJwwmfwBfHWv5OHXMiIlIG08NjjVdrmr0R-TV9bUM</t>
+  </si>
+  <si>
+    <t>Xhaka</t>
+  </si>
+  <si>
+    <t>https://encrypted-tbn2.gstatic.com/licensed-image?q=tbn:ANd9GcTDfW6JR0MouZSoPOFHeTMUCAzqQYIF3ReYOTZxcPBmJn6NDyRuGk34HYGZX9iv7TuncbUTaR8EDFNysNg</t>
+  </si>
+  <si>
+    <t>Jonathan David</t>
+  </si>
+  <si>
+    <t>https://encrypted-tbn2.gstatic.com/licensed-image?q=tbn:ANd9GcQC_13Fkv20dYBrPAd_HKGPXQ1mcivuxRcDU4Uby_iV4cO3LGes9ESLEA4NluFfbCluam_DwDCStGGRolk</t>
+  </si>
+  <si>
+    <t>Saliba</t>
+  </si>
+  <si>
+    <t>https://encrypted-tbn0.gstatic.com/images?q=tbn:ANd9GcS1WQKysFWBPACPheokl2c4655WZkh4Eve-41n-W68uVtXDmbijLPEWsSVFm16VFn4FE2wZqY_tm0gX3_Mj6XVKzXTg-ku-WE3_QzPgPA&amp;s=10</t>
   </si>
   <si>
     <t>TeamName</t>
@@ -530,9 +887,6 @@
     <t>PA</t>
   </si>
   <si>
-    <t>Colombia</t>
-  </si>
-  <si>
     <t>CO</t>
   </si>
   <si>
@@ -551,7 +905,7 @@
     <t>AT</t>
   </si>
   <si>
-    <t>JOR</t>
+    <t>JO</t>
   </si>
   <si>
     <t>SN</t>
@@ -1393,22 +1747,22 @@
         <v>60</v>
       </c>
       <c r="E12" s="2">
-        <v>0.0</v>
+        <v>1.0</v>
       </c>
       <c r="F12" s="2">
-        <v>1.0</v>
+        <v>0.0</v>
       </c>
       <c r="G12" s="1" t="s">
         <v>8</v>
       </c>
       <c r="H12" s="2" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="I12" s="1" t="s">
         <v>51</v>
       </c>
-      <c r="K12" s="2" t="s">
-        <v>62</v>
+      <c r="J12" s="2" t="s">
+        <v>61</v>
       </c>
       <c r="L12" s="2">
         <v>3.0</v>
@@ -1431,10 +1785,10 @@
         <v>46188.0</v>
       </c>
       <c r="C13" s="1" t="s">
+        <v>62</v>
+      </c>
+      <c r="D13" s="1" t="s">
         <v>63</v>
-      </c>
-      <c r="D13" s="1" t="s">
-        <v>64</v>
       </c>
       <c r="E13" s="2">
         <v>5.0</v>
@@ -1446,16 +1800,16 @@
         <v>8</v>
       </c>
       <c r="H13" s="2" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="I13" s="1" t="s">
         <v>56</v>
       </c>
       <c r="J13" s="2" t="s">
+        <v>64</v>
+      </c>
+      <c r="K13" s="2" t="s">
         <v>65</v>
-      </c>
-      <c r="K13" s="2" t="s">
-        <v>66</v>
       </c>
       <c r="L13" s="2">
         <v>0.0</v>
@@ -1478,10 +1832,10 @@
         <v>46188.0</v>
       </c>
       <c r="C14" s="1" t="s">
+        <v>66</v>
+      </c>
+      <c r="D14" s="1" t="s">
         <v>67</v>
-      </c>
-      <c r="D14" s="1" t="s">
-        <v>68</v>
       </c>
       <c r="E14" s="2">
         <v>0.0</v>
@@ -1496,7 +1850,7 @@
         <v>25</v>
       </c>
       <c r="I14" s="1" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="L14" s="2">
         <v>1.0</v>
@@ -1519,10 +1873,10 @@
         <v>46189.0</v>
       </c>
       <c r="C15" s="1" t="s">
+        <v>69</v>
+      </c>
+      <c r="D15" s="1" t="s">
         <v>70</v>
-      </c>
-      <c r="D15" s="1" t="s">
-        <v>71</v>
       </c>
       <c r="E15" s="2">
         <v>1.0</v>
@@ -1537,13 +1891,13 @@
         <v>25</v>
       </c>
       <c r="I15" s="1" t="s">
+        <v>71</v>
+      </c>
+      <c r="J15" s="2" t="s">
         <v>72</v>
       </c>
-      <c r="J15" s="2" t="s">
+      <c r="K15" s="2" t="s">
         <v>73</v>
-      </c>
-      <c r="K15" s="2" t="s">
-        <v>74</v>
       </c>
       <c r="L15" s="2">
         <v>2.0</v>
@@ -1566,10 +1920,10 @@
         <v>46189.0</v>
       </c>
       <c r="C16" s="1" t="s">
+        <v>74</v>
+      </c>
+      <c r="D16" s="1" t="s">
         <v>75</v>
-      </c>
-      <c r="D16" s="1" t="s">
-        <v>76</v>
       </c>
       <c r="E16" s="2">
         <v>1.0</v>
@@ -1584,13 +1938,13 @@
         <v>25</v>
       </c>
       <c r="I16" s="1" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="J16" s="2" t="s">
+        <v>76</v>
+      </c>
+      <c r="K16" s="2" t="s">
         <v>77</v>
-      </c>
-      <c r="K16" s="2" t="s">
-        <v>78</v>
       </c>
       <c r="L16" s="2">
         <v>1.0</v>
@@ -1613,10 +1967,10 @@
         <v>46189.0</v>
       </c>
       <c r="C17" s="1" t="s">
+        <v>78</v>
+      </c>
+      <c r="D17" s="1" t="s">
         <v>79</v>
-      </c>
-      <c r="D17" s="1" t="s">
-        <v>80</v>
       </c>
       <c r="E17" s="2">
         <v>2.0</v>
@@ -1631,13 +1985,13 @@
         <v>25</v>
       </c>
       <c r="I17" s="1" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="J17" s="2" t="s">
+        <v>80</v>
+      </c>
+      <c r="K17" s="2" t="s">
         <v>81</v>
-      </c>
-      <c r="K17" s="2" t="s">
-        <v>82</v>
       </c>
       <c r="L17" s="2">
         <v>1.0</v>
@@ -1660,10 +2014,10 @@
         <v>46190.0</v>
       </c>
       <c r="C18" s="1" t="s">
+        <v>82</v>
+      </c>
+      <c r="D18" s="1" t="s">
         <v>83</v>
-      </c>
-      <c r="D18" s="1" t="s">
-        <v>84</v>
       </c>
       <c r="E18" s="2">
         <v>3.0</v>
@@ -1675,16 +2029,16 @@
         <v>8</v>
       </c>
       <c r="H18" s="2" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="I18" s="1" t="s">
+        <v>84</v>
+      </c>
+      <c r="J18" s="2" t="s">
         <v>85</v>
       </c>
-      <c r="J18" s="2" t="s">
+      <c r="K18" s="2" t="s">
         <v>86</v>
-      </c>
-      <c r="K18" s="2" t="s">
-        <v>87</v>
       </c>
       <c r="L18" s="2">
         <v>0.0</v>
@@ -1707,10 +2061,10 @@
         <v>46190.0</v>
       </c>
       <c r="C19" s="1" t="s">
+        <v>87</v>
+      </c>
+      <c r="D19" s="1" t="s">
         <v>88</v>
-      </c>
-      <c r="D19" s="1" t="s">
-        <v>89</v>
       </c>
       <c r="E19" s="2">
         <v>1.0</v>
@@ -1722,16 +2076,16 @@
         <v>8</v>
       </c>
       <c r="H19" s="2" t="s">
+        <v>88</v>
+      </c>
+      <c r="I19" s="1" t="s">
+        <v>84</v>
+      </c>
+      <c r="J19" s="2" t="s">
         <v>89</v>
       </c>
-      <c r="I19" s="1" t="s">
-        <v>85</v>
-      </c>
-      <c r="J19" s="2" t="s">
+      <c r="K19" s="2" t="s">
         <v>90</v>
-      </c>
-      <c r="K19" s="2" t="s">
-        <v>91</v>
       </c>
       <c r="L19" s="2">
         <v>0.0</v>
@@ -1754,10 +2108,10 @@
         <v>46190.0</v>
       </c>
       <c r="C20" s="1" t="s">
+        <v>91</v>
+      </c>
+      <c r="D20" s="1" t="s">
         <v>92</v>
-      </c>
-      <c r="D20" s="1" t="s">
-        <v>93</v>
       </c>
       <c r="E20" s="2">
         <v>3.0</v>
@@ -1769,13 +2123,13 @@
         <v>8</v>
       </c>
       <c r="H20" s="2" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="I20" s="1" t="s">
+        <v>93</v>
+      </c>
+      <c r="J20" s="2" t="s">
         <v>94</v>
-      </c>
-      <c r="J20" s="2" t="s">
-        <v>95</v>
       </c>
       <c r="L20" s="2">
         <v>0.0</v>
@@ -1798,22 +2152,34 @@
         <v>46190.0</v>
       </c>
       <c r="C21" s="1" t="s">
+        <v>95</v>
+      </c>
+      <c r="D21" s="1" t="s">
         <v>96</v>
       </c>
-      <c r="D21" s="1" t="s">
+      <c r="E21" s="2">
+        <v>3.0</v>
+      </c>
+      <c r="F21" s="2">
+        <v>1.0</v>
+      </c>
+      <c r="G21" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="H21" s="2" t="s">
+        <v>95</v>
+      </c>
+      <c r="I21" s="1" t="s">
+        <v>93</v>
+      </c>
+      <c r="J21" s="2" t="s">
         <v>97</v>
       </c>
-      <c r="G21" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="H21" s="1" t="s">
+      <c r="K21" s="2" t="s">
         <v>98</v>
       </c>
-      <c r="I21" s="1" t="s">
-        <v>94</v>
-      </c>
       <c r="L21" s="2">
-        <v>0.0</v>
+        <v>1.0</v>
       </c>
       <c r="M21" s="2">
         <v>0.0</v>
@@ -1838,20 +2204,32 @@
       <c r="D22" s="1" t="s">
         <v>100</v>
       </c>
+      <c r="E22" s="2">
+        <v>1.0</v>
+      </c>
+      <c r="F22" s="2">
+        <v>1.0</v>
+      </c>
       <c r="G22" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="H22" s="1" t="s">
-        <v>98</v>
+      <c r="H22" s="2" t="s">
+        <v>25</v>
       </c>
       <c r="I22" s="1" t="s">
         <v>101</v>
       </c>
+      <c r="J22" s="2" t="s">
+        <v>102</v>
+      </c>
+      <c r="K22" s="2" t="s">
+        <v>103</v>
+      </c>
       <c r="L22" s="2">
-        <v>0.0</v>
+        <v>1.0</v>
       </c>
       <c r="M22" s="2">
-        <v>0.0</v>
+        <v>1.0</v>
       </c>
       <c r="N22" s="2">
         <v>0.0</v>
@@ -1868,19 +2246,31 @@
         <v>46191.0</v>
       </c>
       <c r="C23" s="1" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="D23" s="1" t="s">
-        <v>103</v>
+        <v>105</v>
+      </c>
+      <c r="E23" s="2">
+        <v>4.0</v>
+      </c>
+      <c r="F23" s="2">
+        <v>2.0</v>
       </c>
       <c r="G23" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="H23" s="1" t="s">
-        <v>98</v>
+      <c r="H23" s="2" t="s">
+        <v>104</v>
       </c>
       <c r="I23" s="1" t="s">
-        <v>104</v>
+        <v>106</v>
+      </c>
+      <c r="J23" s="2" t="s">
+        <v>107</v>
+      </c>
+      <c r="K23" s="2" t="s">
+        <v>108</v>
       </c>
       <c r="L23" s="2">
         <v>0.0</v>
@@ -1903,25 +2293,34 @@
         <v>46191.0</v>
       </c>
       <c r="C24" s="1" t="s">
-        <v>105</v>
+        <v>109</v>
       </c>
       <c r="D24" s="1" t="s">
+        <v>110</v>
+      </c>
+      <c r="E24" s="2">
+        <v>1.0</v>
+      </c>
+      <c r="F24" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G24" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="H24" s="2" t="s">
+        <v>109</v>
+      </c>
+      <c r="I24" s="1" t="s">
         <v>106</v>
       </c>
-      <c r="G24" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="H24" s="1" t="s">
-        <v>98</v>
-      </c>
-      <c r="I24" s="1" t="s">
-        <v>104</v>
+      <c r="J24" s="2" t="s">
+        <v>111</v>
       </c>
       <c r="L24" s="2">
-        <v>0.0</v>
+        <v>1.0</v>
       </c>
       <c r="M24" s="2">
-        <v>0.0</v>
+        <v>2.0</v>
       </c>
       <c r="N24" s="2">
         <v>0.0</v>
@@ -1938,25 +2337,37 @@
         <v>46191.0</v>
       </c>
       <c r="C25" s="1" t="s">
-        <v>107</v>
+        <v>112</v>
       </c>
       <c r="D25" s="1" t="s">
-        <v>108</v>
+        <v>113</v>
+      </c>
+      <c r="E25" s="2">
+        <v>1.0</v>
+      </c>
+      <c r="F25" s="2">
+        <v>3.0</v>
       </c>
       <c r="G25" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="H25" s="1" t="s">
-        <v>98</v>
+      <c r="H25" s="2" t="s">
+        <v>113</v>
       </c>
       <c r="I25" s="1" t="s">
         <v>101</v>
       </c>
+      <c r="J25" s="2" t="s">
+        <v>114</v>
+      </c>
+      <c r="K25" s="2" t="s">
+        <v>115</v>
+      </c>
       <c r="L25" s="2">
-        <v>0.0</v>
+        <v>1.0</v>
       </c>
       <c r="M25" s="2">
-        <v>0.0</v>
+        <v>1.0</v>
       </c>
       <c r="N25" s="2">
         <v>0.0</v>
@@ -1978,20 +2389,32 @@
       <c r="D26" s="1" t="s">
         <v>20</v>
       </c>
+      <c r="E26" s="2">
+        <v>1.0</v>
+      </c>
+      <c r="F26" s="2">
+        <v>1.0</v>
+      </c>
       <c r="G26" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="H26" s="1" t="s">
-        <v>98</v>
+      <c r="H26" s="2" t="s">
+        <v>20</v>
       </c>
       <c r="I26" s="1" t="s">
         <v>17</v>
       </c>
+      <c r="J26" s="2" t="s">
+        <v>116</v>
+      </c>
+      <c r="K26" s="2" t="s">
+        <v>117</v>
+      </c>
       <c r="L26" s="2">
-        <v>0.0</v>
+        <v>2.0</v>
       </c>
       <c r="M26" s="2">
-        <v>0.0</v>
+        <v>1.0</v>
       </c>
       <c r="N26" s="2">
         <v>0.0</v>
@@ -2013,23 +2436,35 @@
       <c r="D27" s="1" t="s">
         <v>35</v>
       </c>
+      <c r="E27" s="2">
+        <v>1.0</v>
+      </c>
+      <c r="F27" s="2">
+        <v>4.0</v>
+      </c>
       <c r="G27" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="H27" s="1" t="s">
-        <v>98</v>
+      <c r="H27" s="2" t="s">
+        <v>35</v>
       </c>
       <c r="I27" s="1" t="s">
         <v>26</v>
       </c>
+      <c r="J27" s="2" t="s">
+        <v>118</v>
+      </c>
+      <c r="K27" s="2" t="s">
+        <v>119</v>
+      </c>
       <c r="L27" s="2">
-        <v>0.0</v>
+        <v>2.0</v>
       </c>
       <c r="M27" s="2">
-        <v>0.0</v>
+        <v>1.0</v>
       </c>
       <c r="N27" s="2">
-        <v>0.0</v>
+        <v>1.0</v>
       </c>
       <c r="O27" s="2">
         <v>0.0</v>
@@ -2048,23 +2483,32 @@
       <c r="D28" s="1" t="s">
         <v>23</v>
       </c>
+      <c r="E28" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="F28" s="2">
+        <v>6.0</v>
+      </c>
       <c r="G28" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="H28" s="1" t="s">
-        <v>98</v>
+      <c r="H28" s="2" t="s">
+        <v>23</v>
       </c>
       <c r="I28" s="1" t="s">
         <v>26</v>
       </c>
+      <c r="K28" s="2" t="s">
+        <v>120</v>
+      </c>
       <c r="L28" s="2">
-        <v>0.0</v>
+        <v>1.0</v>
       </c>
       <c r="M28" s="2">
-        <v>0.0</v>
+        <v>1.0</v>
       </c>
       <c r="N28" s="2">
-        <v>0.0</v>
+        <v>2.0</v>
       </c>
       <c r="O28" s="2">
         <v>0.0</v>
@@ -2083,20 +2527,29 @@
       <c r="D29" s="1" t="s">
         <v>16</v>
       </c>
+      <c r="E29" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="F29" s="2">
+        <v>1.0</v>
+      </c>
       <c r="G29" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="H29" s="1" t="s">
-        <v>98</v>
+      <c r="H29" s="2" t="s">
+        <v>121</v>
       </c>
       <c r="I29" s="1" t="s">
         <v>17</v>
       </c>
+      <c r="K29" s="2" t="s">
+        <v>122</v>
+      </c>
       <c r="L29" s="2">
         <v>0.0</v>
       </c>
       <c r="M29" s="2">
-        <v>0.0</v>
+        <v>2.0</v>
       </c>
       <c r="N29" s="2">
         <v>0.0</v>
@@ -2122,7 +2575,7 @@
         <v>8</v>
       </c>
       <c r="H30" s="1" t="s">
-        <v>98</v>
+        <v>123</v>
       </c>
       <c r="I30" s="1" t="s">
         <v>31</v>
@@ -2157,7 +2610,7 @@
         <v>8</v>
       </c>
       <c r="H31" s="1" t="s">
-        <v>98</v>
+        <v>123</v>
       </c>
       <c r="I31" s="1" t="s">
         <v>40</v>
@@ -2192,7 +2645,7 @@
         <v>8</v>
       </c>
       <c r="H32" s="1" t="s">
-        <v>98</v>
+        <v>123</v>
       </c>
       <c r="I32" s="1" t="s">
         <v>40</v>
@@ -2227,7 +2680,7 @@
         <v>8</v>
       </c>
       <c r="H33" s="1" t="s">
-        <v>98</v>
+        <v>123</v>
       </c>
       <c r="I33" s="1" t="s">
         <v>31</v>
@@ -2256,13 +2709,13 @@
         <v>54</v>
       </c>
       <c r="D34" s="1" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="G34" s="1" t="s">
         <v>8</v>
       </c>
       <c r="H34" s="1" t="s">
-        <v>98</v>
+        <v>123</v>
       </c>
       <c r="I34" s="1" t="s">
         <v>56</v>
@@ -2297,7 +2750,7 @@
         <v>8</v>
       </c>
       <c r="H35" s="1" t="s">
-        <v>98</v>
+        <v>123</v>
       </c>
       <c r="I35" s="1" t="s">
         <v>51</v>
@@ -2332,7 +2785,7 @@
         <v>8</v>
       </c>
       <c r="H36" s="1" t="s">
-        <v>98</v>
+        <v>123</v>
       </c>
       <c r="I36" s="1" t="s">
         <v>51</v>
@@ -2358,7 +2811,7 @@
         <v>46194.0</v>
       </c>
       <c r="C37" s="1" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="D37" s="1" t="s">
         <v>55</v>
@@ -2367,7 +2820,7 @@
         <v>8</v>
       </c>
       <c r="H37" s="1" t="s">
-        <v>98</v>
+        <v>123</v>
       </c>
       <c r="I37" s="1" t="s">
         <v>56</v>
@@ -2393,19 +2846,19 @@
         <v>46194.0</v>
       </c>
       <c r="C38" s="1" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="D38" s="1" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="G38" s="1" t="s">
         <v>8</v>
       </c>
       <c r="H38" s="1" t="s">
-        <v>98</v>
+        <v>123</v>
       </c>
       <c r="I38" s="1" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="L38" s="2">
         <v>0.0</v>
@@ -2428,19 +2881,19 @@
         <v>46195.0</v>
       </c>
       <c r="C39" s="2" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="D39" s="2" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="G39" s="1" t="s">
         <v>8</v>
       </c>
       <c r="H39" s="1" t="s">
-        <v>98</v>
+        <v>123</v>
       </c>
       <c r="I39" s="2" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="L39" s="2">
         <v>0.0</v>
@@ -2463,19 +2916,19 @@
         <v>46195.0</v>
       </c>
       <c r="C40" s="2" t="s">
+        <v>67</v>
+      </c>
+      <c r="D40" s="2" t="s">
+        <v>75</v>
+      </c>
+      <c r="G40" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="H40" s="1" t="s">
+        <v>123</v>
+      </c>
+      <c r="I40" s="2" t="s">
         <v>68</v>
-      </c>
-      <c r="D40" s="2" t="s">
-        <v>76</v>
-      </c>
-      <c r="G40" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="H40" s="1" t="s">
-        <v>98</v>
-      </c>
-      <c r="I40" s="2" t="s">
-        <v>69</v>
       </c>
       <c r="L40" s="2">
         <v>0.0</v>
@@ -2498,19 +2951,19 @@
         <v>46195.0</v>
       </c>
       <c r="C41" s="2" t="s">
+        <v>70</v>
+      </c>
+      <c r="D41" s="2" t="s">
+        <v>79</v>
+      </c>
+      <c r="G41" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="H41" s="1" t="s">
+        <v>123</v>
+      </c>
+      <c r="I41" s="2" t="s">
         <v>71</v>
-      </c>
-      <c r="D41" s="2" t="s">
-        <v>80</v>
-      </c>
-      <c r="G41" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="H41" s="1" t="s">
-        <v>98</v>
-      </c>
-      <c r="I41" s="2" t="s">
-        <v>72</v>
       </c>
       <c r="L41" s="2">
         <v>0.0</v>
@@ -2533,19 +2986,19 @@
         <v>46195.0</v>
       </c>
       <c r="C42" s="2" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="D42" s="2" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="G42" s="1" t="s">
         <v>8</v>
       </c>
       <c r="H42" s="1" t="s">
-        <v>98</v>
+        <v>123</v>
       </c>
       <c r="I42" s="2" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="L42" s="2">
         <v>0.0</v>
@@ -2568,19 +3021,19 @@
         <v>46196.0</v>
       </c>
       <c r="C43" s="2" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="D43" s="2" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="G43" s="1" t="s">
         <v>8</v>
       </c>
       <c r="H43" s="1" t="s">
-        <v>98</v>
+        <v>123</v>
       </c>
       <c r="I43" s="2" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="L43" s="2">
         <v>0.0</v>
@@ -2603,19 +3056,19 @@
         <v>46196.0</v>
       </c>
       <c r="C44" s="2" t="s">
+        <v>83</v>
+      </c>
+      <c r="D44" s="2" t="s">
+        <v>88</v>
+      </c>
+      <c r="G44" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="H44" s="1" t="s">
+        <v>123</v>
+      </c>
+      <c r="I44" s="2" t="s">
         <v>84</v>
-      </c>
-      <c r="D44" s="2" t="s">
-        <v>89</v>
-      </c>
-      <c r="G44" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="H44" s="1" t="s">
-        <v>98</v>
-      </c>
-      <c r="I44" s="2" t="s">
-        <v>85</v>
       </c>
       <c r="L44" s="2">
         <v>0.0</v>
@@ -2638,19 +3091,19 @@
         <v>46196.0</v>
       </c>
       <c r="C45" s="2" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="D45" s="2" t="s">
+        <v>92</v>
+      </c>
+      <c r="G45" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="H45" s="1" t="s">
+        <v>123</v>
+      </c>
+      <c r="I45" s="2" t="s">
         <v>93</v>
-      </c>
-      <c r="G45" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="H45" s="1" t="s">
-        <v>98</v>
-      </c>
-      <c r="I45" s="2" t="s">
-        <v>94</v>
       </c>
       <c r="L45" s="2">
         <v>0.0</v>
@@ -2676,13 +3129,13 @@
         <v>99</v>
       </c>
       <c r="D46" s="2" t="s">
-        <v>107</v>
+        <v>112</v>
       </c>
       <c r="G46" s="1" t="s">
         <v>8</v>
       </c>
       <c r="H46" s="1" t="s">
-        <v>98</v>
+        <v>123</v>
       </c>
       <c r="I46" s="2" t="s">
         <v>101</v>
@@ -2708,19 +3161,19 @@
         <v>46197.0</v>
       </c>
       <c r="C47" s="2" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="D47" s="2" t="s">
-        <v>105</v>
+        <v>109</v>
       </c>
       <c r="G47" s="1" t="s">
         <v>8</v>
       </c>
       <c r="H47" s="1" t="s">
-        <v>98</v>
+        <v>123</v>
       </c>
       <c r="I47" s="2" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="L47" s="2">
         <v>0.0</v>
@@ -2743,19 +3196,19 @@
         <v>46197.0</v>
       </c>
       <c r="C48" s="2" t="s">
+        <v>110</v>
+      </c>
+      <c r="D48" s="2" t="s">
+        <v>105</v>
+      </c>
+      <c r="G48" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="H48" s="1" t="s">
+        <v>123</v>
+      </c>
+      <c r="I48" s="2" t="s">
         <v>106</v>
-      </c>
-      <c r="D48" s="2" t="s">
-        <v>103</v>
-      </c>
-      <c r="G48" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="H48" s="1" t="s">
-        <v>98</v>
-      </c>
-      <c r="I48" s="2" t="s">
-        <v>104</v>
       </c>
       <c r="L48" s="2">
         <v>0.0</v>
@@ -2778,7 +3231,7 @@
         <v>46197.0</v>
       </c>
       <c r="C49" s="2" t="s">
-        <v>108</v>
+        <v>113</v>
       </c>
       <c r="D49" s="2" t="s">
         <v>100</v>
@@ -2787,7 +3240,7 @@
         <v>8</v>
       </c>
       <c r="H49" s="1" t="s">
-        <v>98</v>
+        <v>123</v>
       </c>
       <c r="I49" s="2" t="s">
         <v>101</v>
@@ -2822,7 +3275,7 @@
         <v>8</v>
       </c>
       <c r="H50" s="1" t="s">
-        <v>98</v>
+        <v>123</v>
       </c>
       <c r="I50" s="2" t="s">
         <v>26</v>
@@ -2857,7 +3310,7 @@
         <v>8</v>
       </c>
       <c r="H51" s="1" t="s">
-        <v>98</v>
+        <v>123</v>
       </c>
       <c r="I51" s="2" t="s">
         <v>26</v>
@@ -2892,7 +3345,7 @@
         <v>8</v>
       </c>
       <c r="H52" s="1" t="s">
-        <v>98</v>
+        <v>123</v>
       </c>
       <c r="I52" s="2" t="s">
         <v>40</v>
@@ -2927,7 +3380,7 @@
         <v>8</v>
       </c>
       <c r="H53" s="1" t="s">
-        <v>98</v>
+        <v>123</v>
       </c>
       <c r="I53" s="2" t="s">
         <v>40</v>
@@ -2962,7 +3415,7 @@
         <v>8</v>
       </c>
       <c r="H54" s="1" t="s">
-        <v>98</v>
+        <v>123</v>
       </c>
       <c r="I54" s="2" t="s">
         <v>17</v>
@@ -2997,7 +3450,7 @@
         <v>8</v>
       </c>
       <c r="H55" s="1" t="s">
-        <v>98</v>
+        <v>123</v>
       </c>
       <c r="I55" s="2" t="s">
         <v>17</v>
@@ -3032,7 +3485,7 @@
         <v>8</v>
       </c>
       <c r="H56" s="1" t="s">
-        <v>98</v>
+        <v>123</v>
       </c>
       <c r="I56" s="2" t="s">
         <v>51</v>
@@ -3067,7 +3520,7 @@
         <v>8</v>
       </c>
       <c r="H57" s="1" t="s">
-        <v>98</v>
+        <v>123</v>
       </c>
       <c r="I57" s="2" t="s">
         <v>51</v>
@@ -3093,7 +3546,7 @@
         <v>46199.0</v>
       </c>
       <c r="C58" s="2" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="D58" s="2" t="s">
         <v>54</v>
@@ -3102,7 +3555,7 @@
         <v>8</v>
       </c>
       <c r="H58" s="1" t="s">
-        <v>98</v>
+        <v>123</v>
       </c>
       <c r="I58" s="2" t="s">
         <v>56</v>
@@ -3131,13 +3584,13 @@
         <v>55</v>
       </c>
       <c r="D59" s="2" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="G59" s="1" t="s">
         <v>8</v>
       </c>
       <c r="H59" s="1" t="s">
-        <v>98</v>
+        <v>123</v>
       </c>
       <c r="I59" s="2" t="s">
         <v>56</v>
@@ -3172,7 +3625,7 @@
         <v>8</v>
       </c>
       <c r="H60" s="1" t="s">
-        <v>98</v>
+        <v>123</v>
       </c>
       <c r="I60" s="2" t="s">
         <v>31</v>
@@ -3207,7 +3660,7 @@
         <v>8</v>
       </c>
       <c r="H61" s="1" t="s">
-        <v>98</v>
+        <v>123</v>
       </c>
       <c r="I61" s="2" t="s">
         <v>31</v>
@@ -3233,19 +3686,19 @@
         <v>46200.0</v>
       </c>
       <c r="C62" s="2" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="D62" s="2" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="G62" s="1" t="s">
         <v>8</v>
       </c>
       <c r="H62" s="1" t="s">
-        <v>98</v>
+        <v>123</v>
       </c>
       <c r="I62" s="2" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="L62" s="2">
         <v>0.0</v>
@@ -3268,19 +3721,19 @@
         <v>46200.0</v>
       </c>
       <c r="C63" s="2" t="s">
+        <v>83</v>
+      </c>
+      <c r="D63" s="2" t="s">
+        <v>87</v>
+      </c>
+      <c r="G63" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="H63" s="1" t="s">
+        <v>123</v>
+      </c>
+      <c r="I63" s="2" t="s">
         <v>84</v>
-      </c>
-      <c r="D63" s="2" t="s">
-        <v>88</v>
-      </c>
-      <c r="G63" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="H63" s="1" t="s">
-        <v>98</v>
-      </c>
-      <c r="I63" s="2" t="s">
-        <v>85</v>
       </c>
       <c r="L63" s="2">
         <v>0.0</v>
@@ -3303,19 +3756,19 @@
         <v>46200.0</v>
       </c>
       <c r="C64" s="2" t="s">
+        <v>67</v>
+      </c>
+      <c r="D64" s="2" t="s">
+        <v>74</v>
+      </c>
+      <c r="G64" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="H64" s="1" t="s">
+        <v>123</v>
+      </c>
+      <c r="I64" s="2" t="s">
         <v>68</v>
-      </c>
-      <c r="D64" s="2" t="s">
-        <v>75</v>
-      </c>
-      <c r="G64" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="H64" s="1" t="s">
-        <v>98</v>
-      </c>
-      <c r="I64" s="2" t="s">
-        <v>69</v>
       </c>
       <c r="L64" s="2">
         <v>0.0</v>
@@ -3338,19 +3791,19 @@
         <v>46200.0</v>
       </c>
       <c r="C65" s="2" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="D65" s="2" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="G65" s="1" t="s">
         <v>8</v>
       </c>
       <c r="H65" s="1" t="s">
-        <v>98</v>
+        <v>123</v>
       </c>
       <c r="I65" s="2" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="L65" s="2">
         <v>0.0</v>
@@ -3373,19 +3826,19 @@
         <v>46200.0</v>
       </c>
       <c r="C66" s="2" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="D66" s="2" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="G66" s="1" t="s">
         <v>8</v>
       </c>
       <c r="H66" s="1" t="s">
-        <v>98</v>
+        <v>123</v>
       </c>
       <c r="I66" s="2" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="L66" s="2">
         <v>0.0</v>
@@ -3408,19 +3861,19 @@
         <v>46200.0</v>
       </c>
       <c r="C67" s="2" t="s">
+        <v>70</v>
+      </c>
+      <c r="D67" s="2" t="s">
+        <v>78</v>
+      </c>
+      <c r="G67" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="H67" s="1" t="s">
+        <v>123</v>
+      </c>
+      <c r="I67" s="2" t="s">
         <v>71</v>
-      </c>
-      <c r="D67" s="2" t="s">
-        <v>79</v>
-      </c>
-      <c r="G67" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="H67" s="1" t="s">
-        <v>98</v>
-      </c>
-      <c r="I67" s="2" t="s">
-        <v>72</v>
       </c>
       <c r="L67" s="2">
         <v>0.0</v>
@@ -3443,19 +3896,19 @@
         <v>46201.0</v>
       </c>
       <c r="C68" s="2" t="s">
+        <v>110</v>
+      </c>
+      <c r="D68" s="2" t="s">
+        <v>104</v>
+      </c>
+      <c r="G68" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="H68" s="1" t="s">
+        <v>123</v>
+      </c>
+      <c r="I68" s="2" t="s">
         <v>106</v>
-      </c>
-      <c r="D68" s="2" t="s">
-        <v>102</v>
-      </c>
-      <c r="G68" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="H68" s="1" t="s">
-        <v>98</v>
-      </c>
-      <c r="I68" s="2" t="s">
-        <v>104</v>
       </c>
       <c r="L68" s="2">
         <v>0.0</v>
@@ -3478,19 +3931,19 @@
         <v>46201.0</v>
       </c>
       <c r="C69" s="2" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="D69" s="2" t="s">
-        <v>105</v>
+        <v>109</v>
       </c>
       <c r="G69" s="1" t="s">
         <v>8</v>
       </c>
       <c r="H69" s="1" t="s">
-        <v>98</v>
+        <v>123</v>
       </c>
       <c r="I69" s="2" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="L69" s="2">
         <v>0.0</v>
@@ -3513,7 +3966,7 @@
         <v>46201.0</v>
       </c>
       <c r="C70" s="2" t="s">
-        <v>108</v>
+        <v>113</v>
       </c>
       <c r="D70" s="2" t="s">
         <v>99</v>
@@ -3522,7 +3975,7 @@
         <v>8</v>
       </c>
       <c r="H70" s="1" t="s">
-        <v>98</v>
+        <v>123</v>
       </c>
       <c r="I70" s="2" t="s">
         <v>101</v>
@@ -3551,13 +4004,13 @@
         <v>100</v>
       </c>
       <c r="D71" s="2" t="s">
-        <v>107</v>
+        <v>112</v>
       </c>
       <c r="G71" s="1" t="s">
         <v>8</v>
       </c>
       <c r="H71" s="1" t="s">
-        <v>98</v>
+        <v>123</v>
       </c>
       <c r="I71" s="2" t="s">
         <v>101</v>
@@ -3583,19 +4036,19 @@
         <v>46201.0</v>
       </c>
       <c r="C72" s="2" t="s">
+        <v>92</v>
+      </c>
+      <c r="D72" s="2" t="s">
+        <v>95</v>
+      </c>
+      <c r="G72" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="H72" s="1" t="s">
+        <v>123</v>
+      </c>
+      <c r="I72" s="2" t="s">
         <v>93</v>
-      </c>
-      <c r="D72" s="2" t="s">
-        <v>96</v>
-      </c>
-      <c r="G72" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="H72" s="1" t="s">
-        <v>98</v>
-      </c>
-      <c r="I72" s="2" t="s">
-        <v>94</v>
       </c>
       <c r="L72" s="2">
         <v>0.0</v>
@@ -3618,19 +4071,19 @@
         <v>46201.0</v>
       </c>
       <c r="C73" s="2" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="D73" s="2" t="s">
-        <v>109</v>
+        <v>124</v>
       </c>
       <c r="G73" s="1" t="s">
         <v>8</v>
       </c>
       <c r="H73" s="1" t="s">
-        <v>98</v>
+        <v>123</v>
       </c>
       <c r="I73" s="2" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="L73" s="2">
         <v>0.0</v>
@@ -3653,16 +4106,16 @@
         <v>46202.0</v>
       </c>
       <c r="C74" s="2" t="s">
-        <v>98</v>
+        <v>123</v>
       </c>
       <c r="D74" s="2" t="s">
-        <v>98</v>
+        <v>123</v>
       </c>
       <c r="G74" s="2" t="s">
-        <v>110</v>
+        <v>125</v>
       </c>
       <c r="H74" s="2" t="s">
-        <v>98</v>
+        <v>123</v>
       </c>
       <c r="L74" s="2">
         <v>0.0</v>
@@ -3685,16 +4138,16 @@
         <v>46202.0</v>
       </c>
       <c r="C75" s="2" t="s">
-        <v>98</v>
+        <v>123</v>
       </c>
       <c r="D75" s="2" t="s">
-        <v>98</v>
+        <v>123</v>
       </c>
       <c r="G75" s="2" t="s">
-        <v>110</v>
+        <v>125</v>
       </c>
       <c r="H75" s="2" t="s">
-        <v>98</v>
+        <v>123</v>
       </c>
       <c r="L75" s="2">
         <v>0.0</v>
@@ -3717,16 +4170,16 @@
         <v>46203.0</v>
       </c>
       <c r="C76" s="2" t="s">
-        <v>98</v>
+        <v>123</v>
       </c>
       <c r="D76" s="2" t="s">
-        <v>98</v>
+        <v>123</v>
       </c>
       <c r="G76" s="2" t="s">
-        <v>110</v>
+        <v>125</v>
       </c>
       <c r="H76" s="2" t="s">
-        <v>98</v>
+        <v>123</v>
       </c>
       <c r="L76" s="2">
         <v>0.0</v>
@@ -3749,16 +4202,16 @@
         <v>46203.0</v>
       </c>
       <c r="C77" s="2" t="s">
-        <v>98</v>
+        <v>123</v>
       </c>
       <c r="D77" s="2" t="s">
-        <v>98</v>
+        <v>123</v>
       </c>
       <c r="G77" s="2" t="s">
-        <v>110</v>
+        <v>125</v>
       </c>
       <c r="H77" s="2" t="s">
-        <v>98</v>
+        <v>123</v>
       </c>
       <c r="L77" s="2">
         <v>0.0</v>
@@ -3781,16 +4234,16 @@
         <v>46203.0</v>
       </c>
       <c r="C78" s="2" t="s">
-        <v>98</v>
+        <v>123</v>
       </c>
       <c r="D78" s="2" t="s">
-        <v>98</v>
+        <v>123</v>
       </c>
       <c r="G78" s="2" t="s">
-        <v>110</v>
+        <v>125</v>
       </c>
       <c r="H78" s="2" t="s">
-        <v>98</v>
+        <v>123</v>
       </c>
       <c r="L78" s="2">
         <v>0.0</v>
@@ -3813,16 +4266,16 @@
         <v>46204.0</v>
       </c>
       <c r="C79" s="2" t="s">
-        <v>98</v>
+        <v>123</v>
       </c>
       <c r="D79" s="2" t="s">
-        <v>98</v>
+        <v>123</v>
       </c>
       <c r="G79" s="2" t="s">
-        <v>110</v>
+        <v>125</v>
       </c>
       <c r="H79" s="2" t="s">
-        <v>98</v>
+        <v>123</v>
       </c>
       <c r="L79" s="2">
         <v>0.0</v>
@@ -3845,16 +4298,16 @@
         <v>46204.0</v>
       </c>
       <c r="C80" s="2" t="s">
-        <v>98</v>
+        <v>123</v>
       </c>
       <c r="D80" s="2" t="s">
-        <v>98</v>
+        <v>123</v>
       </c>
       <c r="G80" s="2" t="s">
-        <v>110</v>
+        <v>125</v>
       </c>
       <c r="H80" s="2" t="s">
-        <v>98</v>
+        <v>123</v>
       </c>
       <c r="L80" s="2">
         <v>0.0</v>
@@ -3877,16 +4330,16 @@
         <v>46205.0</v>
       </c>
       <c r="C81" s="2" t="s">
-        <v>98</v>
+        <v>123</v>
       </c>
       <c r="D81" s="2" t="s">
-        <v>98</v>
+        <v>123</v>
       </c>
       <c r="G81" s="2" t="s">
-        <v>110</v>
+        <v>125</v>
       </c>
       <c r="H81" s="2" t="s">
-        <v>98</v>
+        <v>123</v>
       </c>
       <c r="L81" s="2">
         <v>0.0</v>
@@ -3909,16 +4362,16 @@
         <v>46205.0</v>
       </c>
       <c r="C82" s="2" t="s">
-        <v>98</v>
+        <v>123</v>
       </c>
       <c r="D82" s="2" t="s">
-        <v>98</v>
+        <v>123</v>
       </c>
       <c r="G82" s="2" t="s">
-        <v>110</v>
+        <v>125</v>
       </c>
       <c r="H82" s="2" t="s">
-        <v>98</v>
+        <v>123</v>
       </c>
       <c r="L82" s="2">
         <v>0.0</v>
@@ -3941,16 +4394,16 @@
         <v>46205.0</v>
       </c>
       <c r="C83" s="2" t="s">
-        <v>98</v>
+        <v>123</v>
       </c>
       <c r="D83" s="2" t="s">
-        <v>98</v>
+        <v>123</v>
       </c>
       <c r="G83" s="2" t="s">
-        <v>110</v>
+        <v>125</v>
       </c>
       <c r="H83" s="2" t="s">
-        <v>98</v>
+        <v>123</v>
       </c>
       <c r="L83" s="2">
         <v>0.0</v>
@@ -3973,16 +4426,16 @@
         <v>46206.0</v>
       </c>
       <c r="C84" s="2" t="s">
-        <v>98</v>
+        <v>123</v>
       </c>
       <c r="D84" s="2" t="s">
-        <v>98</v>
+        <v>123</v>
       </c>
       <c r="G84" s="2" t="s">
-        <v>110</v>
+        <v>125</v>
       </c>
       <c r="H84" s="2" t="s">
-        <v>98</v>
+        <v>123</v>
       </c>
       <c r="L84" s="2">
         <v>0.0</v>
@@ -4005,16 +4458,16 @@
         <v>46206.0</v>
       </c>
       <c r="C85" s="2" t="s">
-        <v>98</v>
+        <v>123</v>
       </c>
       <c r="D85" s="2" t="s">
-        <v>98</v>
+        <v>123</v>
       </c>
       <c r="G85" s="2" t="s">
-        <v>110</v>
+        <v>125</v>
       </c>
       <c r="H85" s="2" t="s">
-        <v>98</v>
+        <v>123</v>
       </c>
       <c r="L85" s="2">
         <v>0.0</v>
@@ -4037,16 +4490,16 @@
         <v>46206.0</v>
       </c>
       <c r="C86" s="2" t="s">
-        <v>98</v>
+        <v>123</v>
       </c>
       <c r="D86" s="2" t="s">
-        <v>98</v>
+        <v>123</v>
       </c>
       <c r="G86" s="2" t="s">
-        <v>110</v>
+        <v>125</v>
       </c>
       <c r="H86" s="2" t="s">
-        <v>98</v>
+        <v>123</v>
       </c>
       <c r="L86" s="2">
         <v>0.0</v>
@@ -4069,16 +4522,16 @@
         <v>46206.0</v>
       </c>
       <c r="C87" s="2" t="s">
-        <v>98</v>
+        <v>123</v>
       </c>
       <c r="D87" s="2" t="s">
-        <v>98</v>
+        <v>123</v>
       </c>
       <c r="G87" s="2" t="s">
-        <v>110</v>
+        <v>125</v>
       </c>
       <c r="H87" s="2" t="s">
-        <v>98</v>
+        <v>123</v>
       </c>
       <c r="L87" s="2">
         <v>0.0</v>
@@ -4101,16 +4554,16 @@
         <v>46207.0</v>
       </c>
       <c r="C88" s="2" t="s">
-        <v>98</v>
+        <v>123</v>
       </c>
       <c r="D88" s="2" t="s">
-        <v>98</v>
+        <v>123</v>
       </c>
       <c r="G88" s="2" t="s">
-        <v>110</v>
+        <v>125</v>
       </c>
       <c r="H88" s="2" t="s">
-        <v>98</v>
+        <v>123</v>
       </c>
       <c r="L88" s="2">
         <v>0.0</v>
@@ -4133,16 +4586,16 @@
         <v>46207.0</v>
       </c>
       <c r="C89" s="2" t="s">
-        <v>98</v>
+        <v>123</v>
       </c>
       <c r="D89" s="2" t="s">
-        <v>98</v>
+        <v>123</v>
       </c>
       <c r="G89" s="2" t="s">
-        <v>110</v>
+        <v>125</v>
       </c>
       <c r="H89" s="2" t="s">
-        <v>98</v>
+        <v>123</v>
       </c>
       <c r="L89" s="2">
         <v>0.0</v>
@@ -4165,16 +4618,16 @@
         <v>46207.0</v>
       </c>
       <c r="C90" s="2" t="s">
-        <v>98</v>
+        <v>123</v>
       </c>
       <c r="D90" s="2" t="s">
-        <v>98</v>
+        <v>123</v>
       </c>
       <c r="G90" s="2" t="s">
-        <v>111</v>
+        <v>126</v>
       </c>
       <c r="H90" s="2" t="s">
-        <v>98</v>
+        <v>123</v>
       </c>
       <c r="L90" s="2">
         <v>0.0</v>
@@ -4197,16 +4650,16 @@
         <v>46208.0</v>
       </c>
       <c r="C91" s="2" t="s">
-        <v>98</v>
+        <v>123</v>
       </c>
       <c r="D91" s="2" t="s">
-        <v>98</v>
+        <v>123</v>
       </c>
       <c r="G91" s="2" t="s">
-        <v>111</v>
+        <v>126</v>
       </c>
       <c r="H91" s="2" t="s">
-        <v>98</v>
+        <v>123</v>
       </c>
       <c r="L91" s="2">
         <v>0.0</v>
@@ -4229,16 +4682,16 @@
         <v>46209.0</v>
       </c>
       <c r="C92" s="2" t="s">
-        <v>98</v>
+        <v>123</v>
       </c>
       <c r="D92" s="2" t="s">
-        <v>98</v>
+        <v>123</v>
       </c>
       <c r="G92" s="2" t="s">
-        <v>111</v>
+        <v>126</v>
       </c>
       <c r="H92" s="2" t="s">
-        <v>98</v>
+        <v>123</v>
       </c>
       <c r="L92" s="2">
         <v>0.0</v>
@@ -4261,16 +4714,16 @@
         <v>46209.0</v>
       </c>
       <c r="C93" s="2" t="s">
-        <v>98</v>
+        <v>123</v>
       </c>
       <c r="D93" s="2" t="s">
-        <v>98</v>
+        <v>123</v>
       </c>
       <c r="G93" s="2" t="s">
-        <v>111</v>
+        <v>126</v>
       </c>
       <c r="H93" s="2" t="s">
-        <v>98</v>
+        <v>123</v>
       </c>
       <c r="L93" s="2">
         <v>0.0</v>
@@ -4293,16 +4746,16 @@
         <v>46210.0</v>
       </c>
       <c r="C94" s="2" t="s">
-        <v>98</v>
+        <v>123</v>
       </c>
       <c r="D94" s="2" t="s">
-        <v>98</v>
+        <v>123</v>
       </c>
       <c r="G94" s="2" t="s">
-        <v>111</v>
+        <v>126</v>
       </c>
       <c r="H94" s="2" t="s">
-        <v>98</v>
+        <v>123</v>
       </c>
       <c r="L94" s="2">
         <v>0.0</v>
@@ -4325,16 +4778,16 @@
         <v>46210.0</v>
       </c>
       <c r="C95" s="2" t="s">
-        <v>98</v>
+        <v>123</v>
       </c>
       <c r="D95" s="2" t="s">
-        <v>98</v>
+        <v>123</v>
       </c>
       <c r="G95" s="2" t="s">
-        <v>111</v>
+        <v>126</v>
       </c>
       <c r="H95" s="2" t="s">
-        <v>98</v>
+        <v>123</v>
       </c>
       <c r="L95" s="2">
         <v>0.0</v>
@@ -4357,16 +4810,16 @@
         <v>46210.0</v>
       </c>
       <c r="C96" s="2" t="s">
-        <v>98</v>
+        <v>123</v>
       </c>
       <c r="D96" s="2" t="s">
-        <v>98</v>
+        <v>123</v>
       </c>
       <c r="G96" s="2" t="s">
-        <v>111</v>
+        <v>126</v>
       </c>
       <c r="H96" s="2" t="s">
-        <v>98</v>
+        <v>123</v>
       </c>
       <c r="L96" s="2">
         <v>0.0</v>
@@ -4389,16 +4842,16 @@
         <v>46211.0</v>
       </c>
       <c r="C97" s="2" t="s">
-        <v>98</v>
+        <v>123</v>
       </c>
       <c r="D97" s="2" t="s">
-        <v>98</v>
+        <v>123</v>
       </c>
       <c r="G97" s="2" t="s">
-        <v>111</v>
+        <v>126</v>
       </c>
       <c r="H97" s="2" t="s">
-        <v>98</v>
+        <v>123</v>
       </c>
       <c r="L97" s="2">
         <v>0.0</v>
@@ -4421,16 +4874,16 @@
         <v>46213.0</v>
       </c>
       <c r="C98" s="2" t="s">
-        <v>98</v>
+        <v>123</v>
       </c>
       <c r="D98" s="2" t="s">
-        <v>98</v>
+        <v>123</v>
       </c>
       <c r="G98" s="2" t="s">
-        <v>112</v>
+        <v>127</v>
       </c>
       <c r="H98" s="2" t="s">
-        <v>98</v>
+        <v>123</v>
       </c>
       <c r="L98" s="2">
         <v>0.0</v>
@@ -4453,16 +4906,16 @@
         <v>46214.0</v>
       </c>
       <c r="C99" s="2" t="s">
-        <v>98</v>
+        <v>123</v>
       </c>
       <c r="D99" s="2" t="s">
-        <v>98</v>
+        <v>123</v>
       </c>
       <c r="G99" s="2" t="s">
-        <v>112</v>
+        <v>127</v>
       </c>
       <c r="H99" s="2" t="s">
-        <v>98</v>
+        <v>123</v>
       </c>
     </row>
     <row r="100">
@@ -4473,16 +4926,16 @@
         <v>46215.0</v>
       </c>
       <c r="C100" s="2" t="s">
-        <v>98</v>
+        <v>123</v>
       </c>
       <c r="D100" s="2" t="s">
-        <v>98</v>
+        <v>123</v>
       </c>
       <c r="G100" s="2" t="s">
-        <v>112</v>
+        <v>127</v>
       </c>
       <c r="H100" s="2" t="s">
-        <v>98</v>
+        <v>123</v>
       </c>
     </row>
     <row r="101">
@@ -4493,16 +4946,16 @@
         <v>46215.0</v>
       </c>
       <c r="C101" s="2" t="s">
-        <v>98</v>
+        <v>123</v>
       </c>
       <c r="D101" s="2" t="s">
-        <v>98</v>
+        <v>123</v>
       </c>
       <c r="G101" s="2" t="s">
-        <v>112</v>
+        <v>127</v>
       </c>
       <c r="H101" s="2" t="s">
-        <v>98</v>
+        <v>123</v>
       </c>
     </row>
     <row r="102">
@@ -4513,16 +4966,16 @@
         <v>46218.0</v>
       </c>
       <c r="C102" s="2" t="s">
-        <v>98</v>
+        <v>123</v>
       </c>
       <c r="D102" s="2" t="s">
-        <v>98</v>
+        <v>123</v>
       </c>
       <c r="G102" s="2" t="s">
-        <v>113</v>
+        <v>128</v>
       </c>
       <c r="H102" s="2" t="s">
-        <v>98</v>
+        <v>123</v>
       </c>
     </row>
     <row r="103">
@@ -4533,16 +4986,16 @@
         <v>46219.0</v>
       </c>
       <c r="C103" s="2" t="s">
-        <v>98</v>
+        <v>123</v>
       </c>
       <c r="D103" s="2" t="s">
-        <v>98</v>
+        <v>123</v>
       </c>
       <c r="G103" s="2" t="s">
-        <v>113</v>
+        <v>128</v>
       </c>
       <c r="H103" s="2" t="s">
-        <v>98</v>
+        <v>123</v>
       </c>
     </row>
     <row r="104">
@@ -4553,16 +5006,16 @@
         <v>46222.0</v>
       </c>
       <c r="C104" s="2" t="s">
-        <v>98</v>
+        <v>123</v>
       </c>
       <c r="D104" s="2" t="s">
-        <v>98</v>
+        <v>123</v>
       </c>
       <c r="G104" s="2" t="s">
-        <v>114</v>
+        <v>129</v>
       </c>
       <c r="H104" s="2" t="s">
-        <v>98</v>
+        <v>123</v>
       </c>
     </row>
     <row r="105">
@@ -4573,16 +5026,16 @@
         <v>46223.0</v>
       </c>
       <c r="C105" s="2" t="s">
-        <v>98</v>
+        <v>123</v>
       </c>
       <c r="D105" s="2" t="s">
-        <v>98</v>
+        <v>123</v>
       </c>
       <c r="G105" s="2" t="s">
-        <v>115</v>
+        <v>130</v>
       </c>
       <c r="H105" s="2" t="s">
-        <v>98</v>
+        <v>123</v>
       </c>
     </row>
   </sheetData>
@@ -4602,57 +5055,57 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="2" t="s">
-        <v>116</v>
+        <v>131</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>117</v>
+        <v>132</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>118</v>
+        <v>133</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="s">
-        <v>119</v>
+        <v>134</v>
       </c>
       <c r="B2" s="2" t="s">
         <v>16</v>
       </c>
       <c r="C2" s="6" t="s">
-        <v>120</v>
+        <v>135</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="s">
-        <v>121</v>
+        <v>136</v>
       </c>
       <c r="B3" s="2" t="s">
         <v>16</v>
       </c>
       <c r="C3" s="6" t="s">
-        <v>122</v>
+        <v>137</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="s">
-        <v>123</v>
+        <v>138</v>
       </c>
       <c r="B4" s="2" t="s">
         <v>19</v>
       </c>
       <c r="C4" s="6" t="s">
-        <v>124</v>
+        <v>139</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="s">
-        <v>125</v>
+        <v>140</v>
       </c>
       <c r="B5" s="2" t="s">
         <v>19</v>
       </c>
       <c r="C5" s="6" t="s">
-        <v>126</v>
+        <v>141</v>
       </c>
     </row>
     <row r="6">
@@ -4663,7 +5116,7 @@
         <v>20</v>
       </c>
       <c r="C6" s="6" t="s">
-        <v>127</v>
+        <v>142</v>
       </c>
     </row>
     <row r="7">
@@ -4674,7 +5127,7 @@
         <v>23</v>
       </c>
       <c r="C7" s="6" t="s">
-        <v>128</v>
+        <v>143</v>
       </c>
     </row>
     <row r="8">
@@ -4685,15 +5138,18 @@
         <v>24</v>
       </c>
       <c r="C8" s="6" t="s">
-        <v>129</v>
+        <v>144</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="s">
-        <v>130</v>
+        <v>145</v>
       </c>
       <c r="B9" s="2" t="s">
         <v>30</v>
+      </c>
+      <c r="C9" s="6" t="s">
+        <v>146</v>
       </c>
     </row>
     <row r="10">
@@ -4704,29 +5160,700 @@
         <v>30</v>
       </c>
       <c r="C10" s="6" t="s">
-        <v>131</v>
+        <v>147</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="s">
-        <v>132</v>
+        <v>148</v>
       </c>
       <c r="B11" s="2" t="s">
         <v>29</v>
       </c>
       <c r="C11" s="6" t="s">
-        <v>133</v>
+        <v>149</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="s">
-        <v>134</v>
+        <v>150</v>
       </c>
       <c r="B12" s="2" t="s">
         <v>29</v>
       </c>
       <c r="C12" s="6" t="s">
-        <v>135</v>
+        <v>151</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="B13" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="C13" s="6" t="s">
+        <v>152</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="B14" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="C14" s="6" t="s">
+        <v>153</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="s">
+        <v>154</v>
+      </c>
+      <c r="B15" s="2" t="s">
+        <v>91</v>
+      </c>
+      <c r="C15" s="6" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="s">
+        <v>98</v>
+      </c>
+      <c r="B16" s="2" t="s">
+        <v>96</v>
+      </c>
+      <c r="C16" s="6" t="s">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="s">
+        <v>157</v>
+      </c>
+      <c r="B17" s="2" t="s">
+        <v>95</v>
+      </c>
+      <c r="C17" s="6" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="s">
+        <v>159</v>
+      </c>
+      <c r="B18" s="2" t="s">
+        <v>95</v>
+      </c>
+      <c r="C18" s="6" t="s">
+        <v>160</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="s">
+        <v>161</v>
+      </c>
+      <c r="B19" s="2" t="s">
+        <v>96</v>
+      </c>
+      <c r="C19" s="6" t="s">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="B20" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="C20" s="6" t="s">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="B21" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="C21" s="6" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="B22" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="C22" s="6" t="s">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="2" t="s">
+        <v>166</v>
+      </c>
+      <c r="B23" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="C23" s="6" t="s">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="2" t="s">
+        <v>168</v>
+      </c>
+      <c r="B24" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="C24" s="6" t="s">
+        <v>169</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="2" t="s">
+        <v>170</v>
+      </c>
+      <c r="B25" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="C25" s="6" t="s">
+        <v>171</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="2" t="s">
+        <v>172</v>
+      </c>
+      <c r="B26" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="C26" s="6" t="s">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="2" t="s">
+        <v>174</v>
+      </c>
+      <c r="B27" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="C27" s="6" t="s">
+        <v>175</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="2" t="s">
+        <v>176</v>
+      </c>
+      <c r="B28" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="C28" s="6" t="s">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="2" t="s">
+        <v>178</v>
+      </c>
+      <c r="B29" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="C29" s="6" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="2" t="s">
+        <v>180</v>
+      </c>
+      <c r="B30" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="C30" s="6" t="s">
+        <v>181</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="B31" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="C31" s="6" t="s">
+        <v>182</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="2" t="s">
+        <v>183</v>
+      </c>
+      <c r="B32" s="2" t="s">
+        <v>54</v>
+      </c>
+      <c r="C32" s="6" t="s">
+        <v>184</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="2" t="s">
+        <v>185</v>
+      </c>
+      <c r="B33" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="C33" s="6" t="s">
+        <v>186</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="2" t="s">
+        <v>187</v>
+      </c>
+      <c r="B34" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="C34" s="6" t="s">
+        <v>188</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="2" t="s">
+        <v>189</v>
+      </c>
+      <c r="B35" s="2" t="s">
+        <v>54</v>
+      </c>
+      <c r="C35" s="6" t="s">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="2" t="s">
+        <v>61</v>
+      </c>
+      <c r="B36" s="1" t="s">
+        <v>59</v>
+      </c>
+      <c r="C36" s="6" t="s">
+        <v>191</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="2" t="s">
+        <v>192</v>
+      </c>
+      <c r="B37" s="2" t="s">
+        <v>62</v>
+      </c>
+      <c r="C37" s="6" t="s">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="2" t="s">
+        <v>65</v>
+      </c>
+      <c r="B38" s="2" t="s">
+        <v>63</v>
+      </c>
+      <c r="C38" s="6" t="s">
+        <v>194</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="2" t="s">
+        <v>195</v>
+      </c>
+      <c r="B39" s="2" t="s">
+        <v>62</v>
+      </c>
+      <c r="C39" s="6" t="s">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="2" t="s">
+        <v>197</v>
+      </c>
+      <c r="B40" s="2" t="s">
+        <v>62</v>
+      </c>
+      <c r="C40" s="6" t="s">
+        <v>198</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="2" t="s">
+        <v>199</v>
+      </c>
+      <c r="B41" s="2" t="s">
+        <v>62</v>
+      </c>
+      <c r="C41" s="6" t="s">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="2" t="s">
+        <v>201</v>
+      </c>
+      <c r="B42" s="2" t="s">
+        <v>70</v>
+      </c>
+      <c r="C42" s="6" t="s">
+        <v>202</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="2" t="s">
+        <v>73</v>
+      </c>
+      <c r="B43" s="2" t="s">
+        <v>70</v>
+      </c>
+      <c r="C43" s="6" t="s">
+        <v>203</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="2" t="s">
+        <v>76</v>
+      </c>
+      <c r="B44" s="2" t="s">
+        <v>74</v>
+      </c>
+      <c r="C44" s="6" t="s">
+        <v>204</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="2" t="s">
+        <v>77</v>
+      </c>
+      <c r="B45" s="2" t="s">
+        <v>75</v>
+      </c>
+      <c r="C45" s="6" t="s">
+        <v>205</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="2" t="s">
+        <v>206</v>
+      </c>
+      <c r="B46" s="2" t="s">
+        <v>78</v>
+      </c>
+      <c r="C46" s="6" t="s">
+        <v>207</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="2" t="s">
+        <v>208</v>
+      </c>
+      <c r="B47" s="2" t="s">
+        <v>79</v>
+      </c>
+      <c r="C47" s="6" t="s">
+        <v>209</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="2" t="s">
+        <v>210</v>
+      </c>
+      <c r="B48" s="2" t="s">
+        <v>78</v>
+      </c>
+      <c r="C48" s="6" t="s">
+        <v>211</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="2" t="s">
+        <v>212</v>
+      </c>
+      <c r="B49" s="2" t="s">
+        <v>82</v>
+      </c>
+      <c r="C49" s="6" t="s">
+        <v>213</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="2" t="s">
+        <v>86</v>
+      </c>
+      <c r="B50" s="2" t="s">
+        <v>83</v>
+      </c>
+      <c r="C50" s="6" t="s">
+        <v>214</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="2" t="s">
+        <v>215</v>
+      </c>
+      <c r="B51" s="2" t="s">
+        <v>82</v>
+      </c>
+      <c r="C51" s="6" t="s">
+        <v>216</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="2" t="s">
+        <v>89</v>
+      </c>
+      <c r="B52" s="2" t="s">
+        <v>87</v>
+      </c>
+      <c r="C52" s="6" t="s">
+        <v>217</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="2" t="s">
+        <v>218</v>
+      </c>
+      <c r="B53" s="2" t="s">
+        <v>88</v>
+      </c>
+      <c r="C53" s="6" t="s">
+        <v>219</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="2" t="s">
+        <v>220</v>
+      </c>
+      <c r="B54" s="2" t="s">
+        <v>88</v>
+      </c>
+      <c r="C54" s="6" t="s">
+        <v>221</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="2" t="s">
+        <v>103</v>
+      </c>
+      <c r="B55" s="2" t="s">
+        <v>100</v>
+      </c>
+      <c r="C55" s="6" t="s">
+        <v>222</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="2" t="s">
+        <v>102</v>
+      </c>
+      <c r="B56" s="2" t="s">
+        <v>223</v>
+      </c>
+      <c r="C56" s="6" t="s">
+        <v>224</v>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="2" t="s">
+        <v>225</v>
+      </c>
+      <c r="B57" s="2" t="s">
+        <v>105</v>
+      </c>
+      <c r="C57" s="6" t="s">
+        <v>226</v>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="2" t="s">
+        <v>227</v>
+      </c>
+      <c r="B58" s="2" t="s">
+        <v>105</v>
+      </c>
+      <c r="C58" s="6" t="s">
+        <v>228</v>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="2" t="s">
+        <v>229</v>
+      </c>
+      <c r="B59" s="2" t="s">
+        <v>104</v>
+      </c>
+      <c r="C59" s="6" t="s">
+        <v>230</v>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="2" t="s">
+        <v>231</v>
+      </c>
+      <c r="B60" s="2" t="s">
+        <v>104</v>
+      </c>
+      <c r="C60" s="6" t="s">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="2" t="s">
+        <v>233</v>
+      </c>
+      <c r="B61" s="2" t="s">
+        <v>104</v>
+      </c>
+      <c r="C61" s="6" t="s">
+        <v>234</v>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="2" t="s">
+        <v>114</v>
+      </c>
+      <c r="B62" s="2" t="s">
+        <v>112</v>
+      </c>
+      <c r="C62" s="6" t="s">
+        <v>235</v>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="2" t="s">
+        <v>236</v>
+      </c>
+      <c r="B63" s="2" t="s">
+        <v>113</v>
+      </c>
+      <c r="C63" s="6" t="s">
+        <v>237</v>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="2" t="s">
+        <v>238</v>
+      </c>
+      <c r="B64" s="2" t="s">
+        <v>113</v>
+      </c>
+      <c r="C64" s="6" t="s">
+        <v>239</v>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="2" t="s">
+        <v>240</v>
+      </c>
+      <c r="B65" s="2" t="s">
+        <v>113</v>
+      </c>
+      <c r="C65" s="6" t="s">
+        <v>241</v>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="2" t="s">
+        <v>117</v>
+      </c>
+      <c r="B66" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="C66" s="6" t="s">
+        <v>242</v>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="2" t="s">
+        <v>116</v>
+      </c>
+      <c r="B67" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="C67" s="6" t="s">
+        <v>243</v>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="2" t="s">
+        <v>118</v>
+      </c>
+      <c r="B68" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="C68" s="6" t="s">
+        <v>244</v>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="2" t="s">
+        <v>245</v>
+      </c>
+      <c r="B69" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="C69" s="6" t="s">
+        <v>246</v>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="2" t="s">
+        <v>247</v>
+      </c>
+      <c r="B70" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="C70" s="6" t="s">
+        <v>248</v>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" s="2" t="s">
+        <v>249</v>
+      </c>
+      <c r="B71" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="C71" s="6" t="s">
+        <v>250</v>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="2" t="s">
+        <v>251</v>
+      </c>
+      <c r="B72" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="C72" s="6" t="s">
+        <v>252</v>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" s="2" t="s">
+        <v>253</v>
+      </c>
+      <c r="B73" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="C73" s="6" t="s">
+        <v>254</v>
       </c>
     </row>
   </sheetData>
@@ -4738,11 +5865,73 @@
     <hyperlink r:id="rId5" ref="C6"/>
     <hyperlink r:id="rId6" ref="C7"/>
     <hyperlink r:id="rId7" ref="C8"/>
-    <hyperlink r:id="rId8" ref="C10"/>
-    <hyperlink r:id="rId9" ref="C11"/>
-    <hyperlink r:id="rId10" ref="C12"/>
+    <hyperlink r:id="rId8" ref="C9"/>
+    <hyperlink r:id="rId9" ref="C10"/>
+    <hyperlink r:id="rId10" ref="C11"/>
+    <hyperlink r:id="rId11" ref="C12"/>
+    <hyperlink r:id="rId12" ref="C13"/>
+    <hyperlink r:id="rId13" ref="C14"/>
+    <hyperlink r:id="rId14" ref="C15"/>
+    <hyperlink r:id="rId15" ref="C16"/>
+    <hyperlink r:id="rId16" ref="C17"/>
+    <hyperlink r:id="rId17" ref="C18"/>
+    <hyperlink r:id="rId18" ref="C19"/>
+    <hyperlink r:id="rId19" ref="C20"/>
+    <hyperlink r:id="rId20" ref="C21"/>
+    <hyperlink r:id="rId21" ref="C22"/>
+    <hyperlink r:id="rId22" ref="C23"/>
+    <hyperlink r:id="rId23" ref="C24"/>
+    <hyperlink r:id="rId24" ref="C25"/>
+    <hyperlink r:id="rId25" ref="C26"/>
+    <hyperlink r:id="rId26" ref="C27"/>
+    <hyperlink r:id="rId27" ref="C28"/>
+    <hyperlink r:id="rId28" ref="C29"/>
+    <hyperlink r:id="rId29" ref="C30"/>
+    <hyperlink r:id="rId30" ref="C31"/>
+    <hyperlink r:id="rId31" ref="C32"/>
+    <hyperlink r:id="rId32" ref="C33"/>
+    <hyperlink r:id="rId33" ref="C34"/>
+    <hyperlink r:id="rId34" ref="C35"/>
+    <hyperlink r:id="rId35" ref="C36"/>
+    <hyperlink r:id="rId36" ref="C37"/>
+    <hyperlink r:id="rId37" ref="C38"/>
+    <hyperlink r:id="rId38" ref="C39"/>
+    <hyperlink r:id="rId39" ref="C40"/>
+    <hyperlink r:id="rId40" ref="C41"/>
+    <hyperlink r:id="rId41" ref="C42"/>
+    <hyperlink r:id="rId42" ref="C43"/>
+    <hyperlink r:id="rId43" ref="C44"/>
+    <hyperlink r:id="rId44" ref="C45"/>
+    <hyperlink r:id="rId45" ref="C46"/>
+    <hyperlink r:id="rId46" ref="C47"/>
+    <hyperlink r:id="rId47" ref="C48"/>
+    <hyperlink r:id="rId48" ref="C49"/>
+    <hyperlink r:id="rId49" ref="C50"/>
+    <hyperlink r:id="rId50" ref="C51"/>
+    <hyperlink r:id="rId51" ref="C52"/>
+    <hyperlink r:id="rId52" ref="C53"/>
+    <hyperlink r:id="rId53" ref="C54"/>
+    <hyperlink r:id="rId54" ref="C55"/>
+    <hyperlink r:id="rId55" ref="C56"/>
+    <hyperlink r:id="rId56" ref="C57"/>
+    <hyperlink r:id="rId57" ref="C58"/>
+    <hyperlink r:id="rId58" ref="C59"/>
+    <hyperlink r:id="rId59" ref="C60"/>
+    <hyperlink r:id="rId60" ref="C61"/>
+    <hyperlink r:id="rId61" ref="C62"/>
+    <hyperlink r:id="rId62" ref="C63"/>
+    <hyperlink r:id="rId63" ref="C64"/>
+    <hyperlink r:id="rId64" ref="C65"/>
+    <hyperlink r:id="rId65" ref="C66"/>
+    <hyperlink r:id="rId66" ref="C67"/>
+    <hyperlink r:id="rId67" ref="C68"/>
+    <hyperlink r:id="rId68" ref="C69"/>
+    <hyperlink r:id="rId69" ref="C70"/>
+    <hyperlink r:id="rId70" ref="C71"/>
+    <hyperlink r:id="rId71" ref="C72"/>
+    <hyperlink r:id="rId72" ref="C73"/>
   </hyperlinks>
-  <drawing r:id="rId11"/>
+  <drawing r:id="rId73"/>
 </worksheet>
 </file>
 
@@ -4758,13 +5947,13 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="s">
-        <v>136</v>
+        <v>255</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>8</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>137</v>
+        <v>256</v>
       </c>
     </row>
     <row r="2">
@@ -4775,7 +5964,7 @@
         <v>31</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>138</v>
+        <v>257</v>
       </c>
     </row>
     <row r="3">
@@ -4786,7 +5975,7 @@
         <v>17</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>139</v>
+        <v>258</v>
       </c>
     </row>
     <row r="4">
@@ -4797,7 +5986,7 @@
         <v>26</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>140</v>
+        <v>259</v>
       </c>
     </row>
     <row r="5">
@@ -4808,7 +5997,7 @@
         <v>17</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>141</v>
+        <v>260</v>
       </c>
     </row>
     <row r="6">
@@ -4819,7 +6008,7 @@
         <v>17</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>142</v>
+        <v>261</v>
       </c>
     </row>
     <row r="7">
@@ -4830,7 +6019,7 @@
         <v>17</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>143</v>
+        <v>262</v>
       </c>
     </row>
     <row r="8">
@@ -4841,7 +6030,7 @@
         <v>26</v>
       </c>
       <c r="C8" s="1" t="s">
-        <v>144</v>
+        <v>263</v>
       </c>
     </row>
     <row r="9">
@@ -4852,7 +6041,7 @@
         <v>31</v>
       </c>
       <c r="C9" s="1" t="s">
-        <v>145</v>
+        <v>264</v>
       </c>
     </row>
     <row r="10">
@@ -4863,7 +6052,7 @@
         <v>26</v>
       </c>
       <c r="C10" s="1" t="s">
-        <v>146</v>
+        <v>265</v>
       </c>
     </row>
     <row r="11">
@@ -4874,7 +6063,7 @@
         <v>26</v>
       </c>
       <c r="C11" s="1" t="s">
-        <v>147</v>
+        <v>266</v>
       </c>
     </row>
     <row r="12">
@@ -4885,7 +6074,7 @@
         <v>40</v>
       </c>
       <c r="C12" s="1" t="s">
-        <v>148</v>
+        <v>267</v>
       </c>
     </row>
     <row r="13">
@@ -4896,7 +6085,7 @@
         <v>40</v>
       </c>
       <c r="C13" s="1" t="s">
-        <v>149</v>
+        <v>268</v>
       </c>
     </row>
     <row r="14">
@@ -4907,7 +6096,7 @@
         <v>40</v>
       </c>
       <c r="C14" s="1" t="s">
-        <v>150</v>
+        <v>269</v>
       </c>
     </row>
     <row r="15">
@@ -4918,7 +6107,7 @@
         <v>40</v>
       </c>
       <c r="C15" s="1" t="s">
-        <v>151</v>
+        <v>270</v>
       </c>
     </row>
     <row r="16">
@@ -4929,7 +6118,7 @@
         <v>31</v>
       </c>
       <c r="C16" s="1" t="s">
-        <v>152</v>
+        <v>271</v>
       </c>
     </row>
     <row r="17">
@@ -4940,7 +6129,7 @@
         <v>31</v>
       </c>
       <c r="C17" s="1" t="s">
-        <v>153</v>
+        <v>272</v>
       </c>
     </row>
     <row r="18">
@@ -4951,51 +6140,51 @@
         <v>51</v>
       </c>
       <c r="C18" s="1" t="s">
-        <v>154</v>
+        <v>273</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="1" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="B19" s="1" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="C19" s="1" t="s">
-        <v>155</v>
+        <v>274</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="1" t="s">
+        <v>67</v>
+      </c>
+      <c r="B20" s="1" t="s">
         <v>68</v>
       </c>
-      <c r="B20" s="1" t="s">
-        <v>69</v>
-      </c>
       <c r="C20" s="1" t="s">
-        <v>156</v>
+        <v>275</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="1" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="B21" s="1" t="s">
         <v>56</v>
       </c>
       <c r="C21" s="1" t="s">
-        <v>157</v>
+        <v>276</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="1" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="B22" s="1" t="s">
         <v>56</v>
       </c>
       <c r="C22" s="1" t="s">
-        <v>158</v>
+        <v>277</v>
       </c>
     </row>
     <row r="23">
@@ -5006,7 +6195,7 @@
         <v>51</v>
       </c>
       <c r="C23" s="1" t="s">
-        <v>159</v>
+        <v>278</v>
       </c>
     </row>
     <row r="24">
@@ -5017,7 +6206,7 @@
         <v>51</v>
       </c>
       <c r="C24" s="1" t="s">
-        <v>160</v>
+        <v>279</v>
       </c>
     </row>
     <row r="25">
@@ -5028,7 +6217,7 @@
         <v>56</v>
       </c>
       <c r="C25" s="1" t="s">
-        <v>161</v>
+        <v>280</v>
       </c>
     </row>
     <row r="26">
@@ -5039,7 +6228,7 @@
         <v>56</v>
       </c>
       <c r="C26" s="1" t="s">
-        <v>162</v>
+        <v>281</v>
       </c>
     </row>
     <row r="27">
@@ -5050,84 +6239,84 @@
         <v>51</v>
       </c>
       <c r="C27" s="1" t="s">
-        <v>163</v>
+        <v>282</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="1" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="B28" s="1" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="C28" s="1" t="s">
-        <v>164</v>
+        <v>283</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="1" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="B29" s="1" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="C29" s="1" t="s">
-        <v>165</v>
+        <v>284</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="1" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="B30" s="1" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="C30" s="1" t="s">
-        <v>166</v>
+        <v>285</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="1" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="B31" s="1" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="C31" s="1" t="s">
-        <v>167</v>
+        <v>286</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="1" t="s">
-        <v>105</v>
+        <v>109</v>
       </c>
       <c r="B32" s="1" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="C32" s="1" t="s">
-        <v>168</v>
+        <v>287</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="1" t="s">
+        <v>110</v>
+      </c>
+      <c r="B33" s="1" t="s">
         <v>106</v>
       </c>
-      <c r="B33" s="1" t="s">
-        <v>104</v>
-      </c>
       <c r="C33" s="1" t="s">
-        <v>169</v>
+        <v>288</v>
       </c>
     </row>
     <row r="34">
-      <c r="A34" s="1" t="s">
-        <v>170</v>
+      <c r="A34" s="2" t="s">
+        <v>113</v>
       </c>
       <c r="B34" s="1" t="s">
         <v>101</v>
       </c>
       <c r="C34" s="1" t="s">
-        <v>171</v>
+        <v>289</v>
       </c>
     </row>
     <row r="35">
@@ -5138,7 +6327,7 @@
         <v>101</v>
       </c>
       <c r="C35" s="1" t="s">
-        <v>172</v>
+        <v>290</v>
       </c>
     </row>
     <row r="36">
@@ -5149,150 +6338,150 @@
         <v>101</v>
       </c>
       <c r="C36" s="1" t="s">
-        <v>173</v>
+        <v>291</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="1" t="s">
-        <v>107</v>
+        <v>112</v>
       </c>
       <c r="B37" s="1" t="s">
         <v>101</v>
       </c>
       <c r="C37" s="1" t="s">
-        <v>174</v>
+        <v>292</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="B38" s="1" t="s">
         <v>93</v>
       </c>
-      <c r="B38" s="1" t="s">
-        <v>94</v>
-      </c>
       <c r="C38" s="1" t="s">
-        <v>175</v>
+        <v>293</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="1" t="s">
+        <v>95</v>
+      </c>
+      <c r="B39" s="1" t="s">
+        <v>93</v>
+      </c>
+      <c r="C39" s="1" t="s">
+        <v>294</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="2" t="s">
         <v>96</v>
       </c>
-      <c r="B39" s="1" t="s">
-        <v>94</v>
-      </c>
-      <c r="C39" s="1" t="s">
-        <v>176</v>
-      </c>
-    </row>
-    <row r="40">
-      <c r="A40" s="1" t="s">
-        <v>109</v>
-      </c>
       <c r="B40" s="1" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="C40" s="2" t="s">
-        <v>177</v>
+        <v>295</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="1" t="s">
+        <v>83</v>
+      </c>
+      <c r="B41" s="1" t="s">
         <v>84</v>
       </c>
-      <c r="B41" s="1" t="s">
-        <v>85</v>
-      </c>
       <c r="C41" s="1" t="s">
-        <v>178</v>
+        <v>296</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="1" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="B42" s="1" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="C42" s="1" t="s">
-        <v>179</v>
+        <v>297</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="1" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="B43" s="1" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="C43" s="1" t="s">
-        <v>180</v>
+        <v>298</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="1" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="B44" s="1" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="C44" s="1" t="s">
-        <v>181</v>
+        <v>299</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="1" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="B45" s="1" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="C45" s="1" t="s">
-        <v>182</v>
+        <v>300</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="1" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="B46" s="1" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="C46" s="1" t="s">
-        <v>183</v>
+        <v>301</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="1" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="B47" s="1" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="C47" s="1" t="s">
-        <v>184</v>
+        <v>302</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="1" t="s">
+        <v>70</v>
+      </c>
+      <c r="B48" s="1" t="s">
         <v>71</v>
       </c>
-      <c r="B48" s="1" t="s">
-        <v>72</v>
-      </c>
       <c r="C48" s="1" t="s">
-        <v>185</v>
+        <v>303</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="1" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="B49" s="1" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="C49" s="1" t="s">
-        <v>186</v>
+        <v>304</v>
       </c>
     </row>
   </sheetData>

</xml_diff>